<commit_message>
Fix issue with missing CL.
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/output/Complete Analysis - Values Only.xlsx
+++ b/sample-data/sample-run/output/Complete Analysis - Values Only.xlsx
@@ -706,7 +706,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>April 24, 2026 06:33 PM</t>
+          <t>April 24, 2026 07:02 PM</t>
         </is>
       </c>
       <c r="C3" s="3" t="n"/>
@@ -9382,9 +9382,8 @@
       </c>
       <c r="J2" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL eligible (100% developed, fully mature at 287 months). Maturity-Based Weighting: Tail-exposed period (84+ months); primary weight to Paid/Incurred CL. Selection: 100% Chain-Ladder ultimate.
-Eligible methods: Incurred CL (100% developed, CDF = 1.0). Screened methods: None. Diagnostic-Driven Override: None applicable (fully developed). Convergence Check: Single method; no convergence analysis needed. Bayesian Anchoring: No prior provided; CL indication is fully credible. Asymmetric Conservatism: Not applicable (no prior movement). Reasonability Envelope: Period is fully mature and fully developed; no reasonability flags.
-Data quality: No IBNR component (0.0); development is complete. Final selection holds 100% at CL indication.</t>
+          <t>CL 100% (fully developed, CDF=1.0)
+Eligible methods: CL=3,163,773.70, IE=3,163,773.70, BF=3,163,773.70 â€” all converge to the same value. CDF=1.0 means no projection is required; actual incurred equals ultimate. Maturity=287 months (Tail, 84+ mo per framework); CL is primary. IBNR=0 for all methods. Convergence check: trivially passes. Reasonability: fully mature period â€” no flags. No data quality issues.</t>
         </is>
       </c>
     </row>
@@ -9410,19 +9409,18 @@
         <v>2327733.756319999</v>
       </c>
       <c r="G3" s="42" t="n">
-        <v>2904344.26</v>
+        <v>2327733.76</v>
       </c>
       <c r="H3" s="42" t="n">
-        <v>576610.5036800005</v>
+        <v>0.003680000547319651</v>
       </c>
       <c r="I3" s="42" t="n">
-        <v>704698.0319119995</v>
+        <v>128087.5319119995</v>
       </c>
       <c r="J3" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable (NaN). Incurred Expected (IE) available. BF unavailable (NaN). Only method available is Incurred Expected. Maturity-Based Weighting: Late maturity (275 months). At late maturity, CL would be primary (60–100%); IE would be secondary (0–40%). Given CL unavailability, IE becomes sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (not calculated/unavailable), Incurred BF (not available). Diagnostic-Driven Override: None provided (no case adequacy, closure rate, or diagnostics available). Convergence Check: Single method; convergence check not applicable. Bayesian Anchoring: No prior provided. Asymmetric Conservatism: Not applicable (sole method). Reasonability Envelope: Cannot compute IELR without earned premium. IBNR = 576,610.50 (positive, consistent with development expectation at 275 months).
-Data quality: Single method reliance; recommend CL and BF indications for next study to cross-validate IE.</t>
+          <t>CL 100% (fully developed, CDF=1.0)
+Eligible methods: CL=2,327,733.76 (CDF=1.0, IBNR=0), BF=2,327,733.76 (IBNR=0). IE=2,904,344.26 screened out: IE is 25% above actual at full development, meaning the ELR is not consistent with observed experience; when CDF=1.0 the actual incurred IS the ultimate and IE carries zero weight. Maturity=275 months (Tail, 84+ mo). CL primary at full development. Convergence: CL and BF both equal actual. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9448,19 +9446,18 @@
         <v>1778091.575843999</v>
       </c>
       <c r="G4" s="42" t="n">
-        <v>2633272.13</v>
+        <v>1778091.58</v>
       </c>
       <c r="H4" s="42" t="n">
-        <v>855180.5541560005</v>
+        <v>0.00415600067935884</v>
       </c>
       <c r="I4" s="42" t="n">
-        <v>855180.5541560005</v>
+        <v>0.00415600067935884</v>
       </c>
       <c r="J4" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late maturity (263 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 855,180.55 (positive, reasonable for late maturity).
-Data quality: Single method reliance; CL and BF indications needed for validation.</t>
+          <t>CL 100% (fully developed, CDF=1.0)
+Eligible methods: CL=1,778,091.58 (CDF=1.0, IBNR=0), BF=1,778,091.58 (IBNR=0). IE=2,633,272.13 screened out: ELR-based indication is 48% above actual fully-developed losses; at CDF=1.0 the actual is definitive. Maturity=263 months (Tail, 84+ mo). CL primary. Convergence: CL and BF equal actual. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9486,19 +9483,18 @@
         <v>1151324.74736037</v>
       </c>
       <c r="G5" s="42" t="n">
-        <v>1678710.98</v>
+        <v>1146736.49</v>
       </c>
       <c r="H5" s="42" t="n">
-        <v>556096.2493999996</v>
+        <v>24121.75939999963</v>
       </c>
       <c r="I5" s="42" t="n">
-        <v>556096.2493999996</v>
+        <v>24121.75939999963</v>
       </c>
       <c r="J5" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late maturity (251 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 556,096.25 (positive).
-Data quality: Single method reliance; CL and BF validation needed.</t>
+          <t>CL 60%, BF 40% â€” midpoint 1,146,736.49 (tail maturity, near-fully developed)
+Eligible methods: CL=1,142,148.23, BF=1,151,324.75. IE=1,678,711.00 screened out: IE is 47% above CL/BF at 251-month maturity â€” ELR is entirely non-credible at tail; IE receives zero weight. Maturity=251 months (Tail, 84+ mo); CDF=1.0174 (98.3% developed). CL primary (60%), BF secondary (40%) per tail weighting. Convergence check: CL and BF within 0.8% â€” passes Â±2% threshold; selecting midpoint = (1,142,148.23 + 1,151,324.75)/2 = 1,146,736.49. Asymmetric conservatism: BF is marginally higher; midpoint appropriately biases slightly upward from CL. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9524,19 +9520,18 @@
         <v>2282966.477415849</v>
       </c>
       <c r="G6" s="42" t="n">
-        <v>1712285.2</v>
+        <v>2289934.51</v>
       </c>
       <c r="H6" s="42" t="n">
-        <v>-529863.9321160002</v>
+        <v>47785.37788399961</v>
       </c>
       <c r="I6" s="42" t="n">
-        <v>-529863.9321160002</v>
+        <v>47785.37788399961</v>
       </c>
       <c r="J6" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late maturity (239 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −529,863.93 (negative). RED FLAG: Negative IBNR indicates favorable development or estimation error. Actual incurred (2,242,149) &gt; ultimate (1,712,285), implying adverse reversal. This suggests either case reserve decrease or estimate deterioration. Recommend diagnostic review of case adequacy and reserve study timing for this period.
-Data quality: Single method reliance; negative IBNR flags data quality concern. CL and BF indications critical for validation.</t>
+          <t>CL 60%, BF 40% â€” midpoint 2,289,934.51 (tail maturity, near-fully developed)
+Eligible methods: CL=2,296,902.55, BF=2,282,966.48. IE=1,712,285.20 screened out: IE is 25% below CL at 239-month maturity; ELR non-credible at tail. Maturity=239 months (Tail, 84+ mo); CDF=1.02442 (97.6% developed). CL primary (60%), BF secondary (40%). Convergence check: CL and BF within 0.6% â€” passes; midpoint = (2,296,902.55 + 2,282,966.48)/2 = 2,289,934.51. Note: IE-implied IBNR is negative (actual &gt; IE) â€” confirms IE/ELR under-calibration for this year. No data quality flags beyond IE divergence.</t>
         </is>
       </c>
     </row>
@@ -9562,19 +9557,18 @@
         <v>1574310.216423582</v>
       </c>
       <c r="G7" s="42" t="n">
-        <v>1746530.9</v>
+        <v>1571422.3</v>
       </c>
       <c r="H7" s="42" t="n">
-        <v>228894.1073399994</v>
+        <v>53785.50733999955</v>
       </c>
       <c r="I7" s="42" t="n">
-        <v>284389.8721439997</v>
+        <v>109281.2721439998</v>
       </c>
       <c r="J7" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late maturity (227 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 228,894.11 (positive).
-Data quality: Single method reliance; CL and BF validation needed.</t>
+          <t>CL 60%, BF 40% â€” midpoint 1,571,422.30 (tail maturity, near-fully developed)
+Eligible methods: CL=1,568,534.38, BF=1,574,310.22. IE=1,746,530.90 screened out: IE is 11% above CL at 227-month maturity; ELR non-credible at tail. Maturity=227 months (Tail, 84+ mo); CDF=1.03354 (96.8% developed). CL primary (60%), BF secondary (40%). Convergence check: CL and BF within 0.4% â€” passes; midpoint = (1,568,534.38 + 1,574,310.22)/2 = 1,571,422.30. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9600,19 +9594,18 @@
         <v>4903265.642420489</v>
       </c>
       <c r="G8" s="42" t="n">
-        <v>2850338.44</v>
+        <v>4937690.56</v>
       </c>
       <c r="H8" s="42" t="n">
-        <v>-1960436.174816</v>
+        <v>126915.9451839998</v>
       </c>
       <c r="I8" s="42" t="n">
-        <v>-1940354.713152</v>
+        <v>146997.4068479994</v>
       </c>
       <c r="J8" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late maturity (215 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −1,960,436.18 (large negative). RED FLAG: Very large negative IBNR (actual 4,810,775 &gt;&gt; ultimate 2,850,338). Adverse case development or severe estimation error. This period likely had reserve strengthening after the IE estimate or case reactivations. Recommend diagnostic investigation before finalizing selection.
-Data quality: Single method reliance; large negative IBNR is a material data quality flag. CL and BF indications essential for validation.</t>
+          <t>CL 60%, BF 40% â€” midpoint 4,937,690.56 (tail maturity, near-fully developed)
+Eligible methods: CL=4,972,115.48, BF=4,903,265.64. IE=2,850,338.44 screened out: IE is 43% below CL â€” entirely non-credible at 215-month maturity; the ELR appears calibrated to a much lower loss level. Maturity=215 months (Tail, 84+ mo); CDF=1.03354 (96.8% developed). CL primary (60%), BF secondary (40%). Convergence check: CL and BF within 1.4% â€” passes; midpoint = (4,972,115.48 + 4,903,265.64)/2 = 4,937,690.56. Flag: This period shows unusually elevated losses relative to adjacent years (2006: ~1.6M, 2008: ~1.4M). CL and BF both project elevated ultimates consistently, supporting the selection. The large negative IE IBNR (-1,960,436) confirms IE severely underestimates this year. Data quality flag: elevated loss year; recommend review of individual large claims.</t>
         </is>
       </c>
     </row>
@@ -9638,19 +9631,18 @@
         <v>1465889.113446933</v>
       </c>
       <c r="G9" s="42" t="n">
-        <v>2543927.05</v>
+        <v>1446697.63</v>
       </c>
       <c r="H9" s="42" t="n">
-        <v>1165499.110452001</v>
+        <v>68269.69045200152</v>
       </c>
       <c r="I9" s="42" t="n">
-        <v>1165499.110452001</v>
+        <v>68269.69045200152</v>
       </c>
       <c r="J9" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late maturity (203 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 1,165,499.11 (positive).
-Data quality: Single method reliance; CL and BF validation needed.</t>
+          <t>CL 55%, BF 45% â€” midpoint 1,446,697.63 (tail maturity, 3.6% residual development)
+Eligible methods: CL=1,427,506.14, BF=1,465,889.11. IE=2,543,927.05 screened out: IE is 78% above CL at 203-month maturity â€” non-credible at tail. Maturity=203 months (Tail, 84+ mo); CDF=1.03560 (96.6% developed). CL primary (55%), BF secondary (45%). CL and BF within 2.7% â€” just outside Â±2% convergence; midpoint = (1,427,506.14 + 1,465,889.11)/2 = 1,446,697.63. Asymmetric conservatism: BF is higher; midpoint biases upward from CL. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9676,19 +9668,18 @@
         <v>1277690.378550072</v>
       </c>
       <c r="G10" s="42" t="n">
-        <v>2594805.59</v>
+        <v>1249059.54</v>
       </c>
       <c r="H10" s="42" t="n">
-        <v>1425224.500743999</v>
+        <v>79478.45074399957</v>
       </c>
       <c r="I10" s="42" t="n">
-        <v>1425224.500743999</v>
+        <v>79478.45074399957</v>
       </c>
       <c r="J10" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late maturity (191 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 1,425,224.51 (positive).
-Data quality: Single method reliance; CL and BF validation needed.</t>
+          <t>CL 50%, BF 50% â€” midpoint 1,249,059.54 (tail maturity, 4.3% residual development)
+Eligible methods: CL=1,220,428.71, BF=1,277,690.38. IE=2,594,805.59 screened out: IE is 113% above CL â€” completely non-credible at 191-month maturity. Maturity=191 months (Tail, 84+ mo); CDF=1.04348 (95.8% developed). CL primary but BF retains credibility given WC long-tail adjustment (BF credible longer). CL and BF diverge by 4.7% â€” outside Â±2% convergence. Asymmetric conservatism: BF is higher; upward moves travel farther â€” increase BF weight. Weighted = 0.50*1,220,428.71 + 0.50*1,277,690.38 = 1,249,059.54; midpoint selected as balanced conservative compromise. Flag: IE/ELR implies more than double the CL indication â€” ELR appears severely mis-calibrated for this period.</t>
         </is>
       </c>
     </row>
@@ -9714,19 +9705,18 @@
         <v>1328830.587656843</v>
       </c>
       <c r="G11" s="42" t="n">
-        <v>1134300.73</v>
+        <v>1333424.57</v>
       </c>
       <c r="H11" s="42" t="n">
-        <v>-143371.3420840006</v>
+        <v>55752.4979159995</v>
       </c>
       <c r="I11" s="42" t="n">
-        <v>-143371.3420840006</v>
+        <v>55752.4979159995</v>
       </c>
       <c r="J11" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late-to-mid maturity (179 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −143,371.34 (negative). Actual (1,277,672) &gt; ultimate (1,134,301), indicating adverse development post-estimate. Flag for diagnostic review.
-Data quality: Single method reliance; negative IBNR flags data quality concern. CL and BF indications critical.</t>
+          <t>CL 60%, BF 40% â€” midpoint 1,333,424.57 (tail maturity, 4.7% residual development)
+Eligible methods: CL=1,338,018.54, BF=1,328,830.59. IE=1,134,300.73 screened out: IE is 15% below CL at 179-month maturity; ELR non-credible at tail. Maturity=179 months (Tail, 84+ mo); CDF=1.04723 (95.5% developed). CL primary (60%), BF secondary (40%). Convergence check: CL and BF within 0.7% â€” passes; midpoint = (1,338,018.54 + 1,328,830.59)/2 = 1,333,424.57. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9752,19 +9742,18 @@
         <v>2016096.735607065</v>
       </c>
       <c r="G12" s="42" t="n">
-        <v>1542648.99</v>
+        <v>2032508.37</v>
       </c>
       <c r="H12" s="42" t="n">
-        <v>-373432.5904159998</v>
+        <v>116426.7895840004</v>
       </c>
       <c r="I12" s="42" t="n">
-        <v>-350009.3077319998</v>
+        <v>139850.0722680003</v>
       </c>
       <c r="J12" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Late-to-mid maturity (167 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −373,432.59 (negative). Actual (1,916,082) &gt; ultimate (1,542,649). Adverse development signal. Recommend diagnostic investigation.
-Data quality: Single method reliance; negative IBNR flags data quality. CL and BF validation essential.</t>
+          <t>CL 60%, BF 40% â€” midpoint 2,032,508.37 (tail maturity, 6.9% residual development)
+Eligible methods: CL=2,048,920.00, BF=2,016,096.74. IE=1,542,649.00 screened out: IE is 25% below CL at 167-month maturity; non-credible at tail. Maturity=167 months (Tail, 84+ mo); CDF=1.06933 (93.5% developed). CL primary (60%), BF secondary (40%). Convergence check: CL and BF within 1.6% â€” passes; midpoint = (2,048,920.00 + 2,016,096.74)/2 = 2,032,508.37. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9790,19 +9779,18 @@
         <v>1466357.198096881</v>
       </c>
       <c r="G13" s="42" t="n">
-        <v>1573501.97</v>
+        <v>1462620.21</v>
       </c>
       <c r="H13" s="42" t="n">
-        <v>209748.5894680009</v>
+        <v>98866.82946800091</v>
       </c>
       <c r="I13" s="42" t="n">
-        <v>379265.0916600011</v>
+        <v>268383.3316600011</v>
       </c>
       <c r="J13" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Mid maturity (155 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 209,748.59 (positive).
-Data quality: Single method reliance; CL and BF validation needed.</t>
+          <t>CL 60%, BF 40% â€” midpoint 1,462,620.21 (tail maturity, 7.0% residual development)
+Eligible methods: CL=1,458,883.22, BF=1,466,357.20. IE=1,573,501.97 screened out: IE is 7.7% above CL at 155-month maturity; ELR carries no weight at tail. Maturity=155 months (Tail, 84+ mo); CDF=1.06976 (93.5% developed). CL primary (60%), BF secondary (40%). Convergence check: CL and BF within 0.5% â€” passes; midpoint = (1,458,883.22 + 1,466,357.20)/2 = 1,462,620.21. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9828,19 +9816,18 @@
         <v>789491.9986882674</v>
       </c>
       <c r="G14" s="42" t="n">
-        <v>1203729.01</v>
+        <v>774556.8199999999</v>
       </c>
       <c r="H14" s="42" t="n">
-        <v>495199.0191400001</v>
+        <v>66026.82914000005</v>
       </c>
       <c r="I14" s="42" t="n">
-        <v>495199.0191400001</v>
+        <v>66026.82914000005</v>
       </c>
       <c r="J14" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Mid maturity (143 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 495,199.02 (positive).
-Data quality: Single method reliance; CL and BF validation needed.</t>
+          <t>CL 50%, BF 50% â€” midpoint 774,556.82 (tail maturity, 7.2% residual development)
+Eligible methods: CL=759,621.63, BF=789,492.00. IE=1,203,729.01 screened out: IE is 58% above CL at 143-month maturity â€” completely non-credible at tail. Maturity=143 months (Tail, 84+ mo); CDF=1.07211 (93.3% developed). CL and BF diverge by 3.9% â€” outside Â±2% convergence. Asymmetric conservatism: BF is higher; upward moves travel farther â€” equal weight applied as compromise. Midpoint = (759,621.63 + 789,492.00)/2 = 774,556.82. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9866,19 +9853,18 @@
         <v>1510912.258315372</v>
       </c>
       <c r="G15" s="42" t="n">
-        <v>1227803.59</v>
+        <v>1526431.31</v>
       </c>
       <c r="H15" s="42" t="n">
-        <v>-161800.094732</v>
+        <v>136827.6252679999</v>
       </c>
       <c r="I15" s="42" t="n">
-        <v>-161800.094732</v>
+        <v>136827.6252679999</v>
       </c>
       <c r="J15" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Mid maturity (131 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −161,800.09 (negative). Actual (1,389,604) &gt; ultimate (1,227,804). Adverse post-estimate development. Flag for review.
-Data quality: Single method reliance; negative IBNR flags data quality. CL and BF validation critical.</t>
+          <t>CL 55%, BF 45% â€” midpoint 1,526,431.31 (tail maturity, 11.0% residual development)
+Eligible methods: CL=1,541,950.36, BF=1,510,912.26. IE=1,227,803.59 screened out: IE is 20% below CL at 131-month maturity; non-credible at tail. Maturity=131 months (Tail, 84+ mo); CDF=1.10963 (90.1% developed). CL primary (55%), BF secondary (45%). Convergence check: CL and BF within 2.0% â€” at boundary; midpoint = (1,541,950.36 + 1,510,912.26)/2 = 1,526,431.31. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9904,19 +9890,18 @@
         <v>3560182.188573404</v>
       </c>
       <c r="G16" s="42" t="n">
-        <v>1669812.88</v>
+        <v>3672406.02</v>
       </c>
       <c r="H16" s="42" t="n">
-        <v>-1713150.378076002</v>
+        <v>289442.7619239986</v>
       </c>
       <c r="I16" s="42" t="n">
-        <v>-1694418.418548001</v>
+        <v>308174.7214519987</v>
       </c>
       <c r="J16" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Early-to-mid maturity (119 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −1,713,150.37 (very large negative). RED FLAG: Actual (3,382,963) &gt;&gt; ultimate (1,669,813). Massive adverse development post-estimate. This indicates either: (1) severe IE underestimate, (2) case reserve reactivation, or (3) reopen activity. This period requires immediate diagnostic investigation before finalization. Potential implications for loss control or underwriting.
-Data quality: Single method reliance; very large negative IBNR is a critical data quality flag. CL and BF indications ESSENTIAL. Do not finalize without peer review.</t>
+          <t>CL 55%, BF 45% â€” midpoint 3,672,406.02 (tail maturity, 11.9% residual development)
+Eligible methods: CL=3,784,629.85, BF=3,560,182.19. IE=1,669,812.88 screened out: IE is 56% below CL at 119-month maturity â€” entirely non-credible at tail (ELR severely under-calibrated for this year). Maturity=119 months (Tail, 84+ mo); CDF=1.11873 (89.4% developed). CL primary (55%), BF secondary (45%). CL and BF diverge by 6.3% â€” outside Â±2% convergence. Asymmetric conservatism: CL is higher; upward moves travel farther â€” CL weight maintained at 55%. Midpoint = (3,784,629.85 + 3,560,182.19)/2 = 3,672,406.02. Flag: This period shows notably elevated losses (CL 3.78M vs. neighbors 2014: 1.54M, 2016: 2.96M). CL and BF both confirm elevated ultimate; IE/ELR provides no plausible alternative. Recommend review of large individual claims. The large negative IE IBNR (-1,713,150) confirms IE grossly underestimates this year.</t>
         </is>
       </c>
     </row>
@@ -9942,19 +9927,18 @@
         <v>2900209.319415499</v>
       </c>
       <c r="G17" s="42" t="n">
-        <v>2554813.71</v>
+        <v>2931688.02</v>
       </c>
       <c r="H17" s="42" t="n">
-        <v>48490.0666320012</v>
+        <v>425364.3766320013</v>
       </c>
       <c r="I17" s="42" t="n">
-        <v>92605.03360800119</v>
+        <v>469479.3436080012</v>
       </c>
       <c r="J17" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Early-to-mid maturity (107 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 48,490.07 (positive, small).
-Data quality: Single method reliance; CL and BF validation needed.</t>
+          <t>CL 55%, BF 45% â€” midpoint 2,931,688.02 (tail maturity, 18.2% residual development)
+Eligible methods: CL=2,963,166.71, BF=2,900,209.32. IE=2,554,813.71 screened out: IE is 14% below CL at 107-month maturity; ELR non-credible at tail. Maturity=107 months (Tail, 84+ mo); CDF=1.18228 (84.6% developed). CL primary (55%), BF secondary (45%). Convergence check: CL and BF within 2.2% â€” just outside Â±2% threshold; midpoint = (2,963,166.71 + 2,900,209.32)/2 = 2,931,688.02. Asymmetric conservatism: CL is higher; midpoint appropriately biases upward. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -9980,19 +9964,18 @@
         <v>1639292.683786481</v>
       </c>
       <c r="G18" s="42" t="n">
-        <v>2605909.99</v>
+        <v>1542854.53</v>
       </c>
       <c r="H18" s="42" t="n">
-        <v>1400098.161084</v>
+        <v>337042.7010839996</v>
       </c>
       <c r="I18" s="42" t="n">
-        <v>1400098.161084</v>
+        <v>337042.7010839996</v>
       </c>
       <c r="J18" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Early maturity (95 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 1,400,098.16 (positive).
-Data quality: Single method reliance; CL and BF validation needed.</t>
+          <t>CL 45%, BF 55% â€” midpoint 1,542,854.53 (tail/late boundary, 20.0% residual development)
+Eligible methods: CL=1,446,416.38, BF=1,639,292.68. IE=2,605,909.99 screened out: IE is 80% above CL at 95-month maturity â€” entirely non-credible; the ELR is clearly not representative of this year's actual loss level. Maturity=95 months (Tail, 84+ mo per framework); CDF=1.19954 (83.4% developed). At 95 months with significant residual development (20%), WC long-tail adjustment increases BF weight: BF primary (55%), CL secondary (45%). CL and BF diverge by 13.3% â€” well outside Â±2% convergence. Asymmetric conservatism: BF is higher; upward moves travel farther â€” BF weight maintained at 55%. Weighted = 0.45*1,446,416.38 + 0.55*1,639,292.68 = 650,887.37 + 901,611.0 = 1,552,498; midpoint = (1,446,416.38 + 1,639,292.68)/2 = 1,542,854.53. Selecting midpoint for balance; midpoint is between weighted (1,552,498) and CL-weighted (1,543K). Flag: IE implies 2.6M ultimate vs CL 1.45M â€” very large ELR divergence; ELR excluded.</t>
         </is>
       </c>
     </row>
@@ -10018,19 +10001,18 @@
         <v>2777835.189014538</v>
       </c>
       <c r="G19" s="42" t="n">
-        <v>2215023.49</v>
+        <v>2836551.62</v>
       </c>
       <c r="H19" s="42" t="n">
-        <v>-180424.9333040006</v>
+        <v>441103.1966959992</v>
       </c>
       <c r="I19" s="42" t="n">
-        <v>-180424.9333040006</v>
+        <v>441103.1966959992</v>
       </c>
       <c r="J19" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Early maturity (83 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −180,424.94 (negative). Actual (2,395,448) &gt; ultimate (2,215,023). Adverse development. Flag for review.
-Data quality: Single method reliance; negative IBNR flags data quality. CL validation important.</t>
+          <t>CL 50%, BF 50% â€” midpoint 2,836,551.62 (late maturity, 20.9% residual development)
+Eligible methods: CL=2,895,268.04, BF=2,777,835.19. IE=2,215,023.49 screened out: IE is 23% below CL at 83-month maturity; ELR non-credible at late maturity. Maturity=83 months (Late, 60-84 mo); CDF=1.20865 (82.7% developed). Per late maturity table, CL is primary and BF is secondary; at the upper boundary of late (83 months), BF retains meaningful weight. CL and BF diverge by 4.2% â€” outside Â±2%. Asymmetric conservatism: CL is higher; upward bias applied, equal weighting as compromise. Midpoint = (2,895,268.04 + 2,777,835.19)/2 = 2,836,551.62. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -10056,19 +10038,18 @@
         <v>3139529.318974986</v>
       </c>
       <c r="G20" s="42" t="n">
-        <v>2259323.96</v>
+        <v>3277636.52</v>
       </c>
       <c r="H20" s="42" t="n">
-        <v>-340558.9142919993</v>
+        <v>677753.6457080008</v>
       </c>
       <c r="I20" s="42" t="n">
-        <v>-135865.8744880008</v>
+        <v>882446.6855119993</v>
       </c>
       <c r="J20" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Early maturity (71 months). IE is sole eligible method. Selection: 100% Incurred Expected.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −340,558.92 (negative). Actual (2,599,883) &gt; ultimate (2,259,324). Adverse post-estimate development. Flag for review.
-Data quality: Single method reliance; negative IBNR flags data quality. CL validation critical.</t>
+          <t>CL 40%, BF 60% â€” midpoint 3,277,636.52 (late maturity, 31.4% residual development)
+Eligible methods: CL=3,415,743.72, BF=3,139,529.32. IE=2,259,323.96 screened out: IE is 34% below CL at 71-month maturity; ELR non-credible at late maturity. Maturity=71 months (Late, 60-84 mo); CDF=1.31381 (76.1% developed). At 71 months with 31% residual development, WC long-tail adjustment gives BF primary weight (60%), CL secondary (40%). CL and BF diverge by 8.8% â€” outside Â±2% convergence. Asymmetric conservatism: CL is higher; upward bias applied but BF credibility limits full CL reliance. Midpoint = (3,415,743.72 + 3,139,529.32)/2 = 3,277,636.52. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -10094,19 +10075,18 @@
         <v>1549943.380235656</v>
       </c>
       <c r="G21" s="42" t="n">
-        <v>1843608.35</v>
+        <v>1484054.54</v>
       </c>
       <c r="H21" s="42" t="n">
-        <v>864708.8405320002</v>
+        <v>505155.0305320001</v>
       </c>
       <c r="I21" s="42" t="n">
-        <v>867557.4874440002</v>
+        <v>508003.6774440001</v>
       </c>
       <c r="J21" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Green maturity (59 months). At this maturity, CL is weak (1–20%) and BF is primary (50–70%). Given unavailability, IE is sole method. Selection: 100% Incurred Expected with high uncertainty.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 864,708.84 (positive, represents 47% of ultimate; reasonable for 59-month maturity but signals high remaining exposure). CL and BF indications critical for green period validation.
-Data quality: Single method reliance at early maturity; CL and BF indications CRITICAL. Recommend re-running analysis with BF a priori and CL development.</t>
+          <t>CL 35%, BF 65% â€” midpoint 1,484,054.54 (mid maturity, 31.0% residual development)
+Eligible methods: CL=1,418,165.71, BF=1,549,943.38. IE=1,843,608.35 (secondary, limited weight). Maturity=59 months (Mid, 36-60 mo); CDF=1.44873 (69.0% developed). At mid maturity, CL is primary per framework; however WC long-tail adjustment shifts BF credibility later â€” BF retains substantial weight (65%), CL secondary (35%). IE is 30% above CL and 19% above BF; IE receives minimal weight at mid maturity. CL and BF diverge by 9.3% â€” outside Â±2% convergence. Asymmetric conservatism: BF is higher; upward bias favors BF. Midpoint = (1,418,165.71 + 1,549,943.38)/2 = 1,484,054.54. Reasonability: 2020 losses appear low relative to neighbors (2019: 3.28M, 2021: 1.51M); possible COVID-19 impact on claim activity â€” consistent with observed pattern. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -10132,19 +10112,18 @@
         <v>1493193.146184722</v>
       </c>
       <c r="G22" s="42" t="n">
-        <v>1410360.39</v>
+        <v>1514688.18</v>
       </c>
       <c r="H22" s="42" t="n">
-        <v>399047.1102639999</v>
+        <v>503374.9002639999</v>
       </c>
       <c r="I22" s="42" t="n">
-        <v>435380.9766639997</v>
+        <v>539708.7666639998</v>
       </c>
       <c r="J22" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Green maturity (47 months). At this maturity, BF is primary (70–100%); CL is weak (0–20%). Given unavailability, IE is sole method. Selection: 100% Incurred Expected with high uncertainty.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 399,047.11 (positive, represents 28% of ultimate; reasonable for 47-month maturity). BF a priori and CL development needed.
-Data quality: Single method reliance at very green period; CL and BF validation ESSENTIAL. Re-run with a priori loss ratio and full triangles.</t>
+          <t>CL 35%, BF 65% â€” midpoint 1,514,688.18 (mid maturity, 34.2% residual development)
+Eligible methods: CL=1,536,183.21, BF=1,493,193.15. IE=1,410,360.39 (secondary, limited weight at this maturity). Maturity=47 months (Mid, 36-60 mo); CDF=1.51900 (65.8% developed). WC long-tail: BF retains primary weight (65%), CL secondary (35%). IE is 8.2% below CL â€” minor divergence; IE receives no material weight. CL and BF within 2.9% â€” near convergence boundary. Midpoint = (1,536,183.21 + 1,493,193.15)/2 = 1,514,688.18. Asymmetric conservatism: CL is marginally higher; midpoint appropriate. No data quality flags.</t>
         </is>
       </c>
     </row>
@@ -10170,19 +10149,18 @@
         <v>1260409.883332667</v>
       </c>
       <c r="G23" s="42" t="n">
-        <v>959045.0600000001</v>
+        <v>1384436.85</v>
       </c>
       <c r="H23" s="42" t="n">
-        <v>131628.9533559993</v>
+        <v>557020.7433559994</v>
       </c>
       <c r="I23" s="42" t="n">
-        <v>167941.349864</v>
+        <v>593333.139864</v>
       </c>
       <c r="J23" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Very green maturity (35 months). At this maturity, a priori and BF are primary (70–100%); CL is not credible (0–10%). Given unavailability, IE is sole method. Selection: 100% Incurred Expected with very high uncertainty.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 131,628.96 (positive, represents 14% of ultimate; reasonable for 35-month maturity). BF a priori CRITICAL for this green period.
-Data quality: Single method reliance at very green period; CL and BF data missing. BF a priori and full triangles MANDATORY for next study.</t>
+          <t>BF 70%, CL 30% â€” midpoint 1,384,436.85 (early maturity, 45.1% residual development)
+Eligible methods: CL=1,508,463.82, BF=1,260,409.88. IE=959,045.06 screened out: IE is 36% below CL at 35-month maturity â€” IE/ELR appears severely under-calibrated for this year and receives no weight. Maturity=35 months (Early, 24-36 mo); CDF=1.82310 (54.9% developed). Per early maturity table, BF/CL/Benktander are eligible; BF gets primary weight (70%) and CL secondary (30%) for WC long-tail. At 45% IBNR proportion, CL is applying significant tail leverage â€” BF moderates through ELR blend. CL and BF diverge by 19.7% â€” large gap expected at early maturity. Asymmetric conservatism: CL is higher; upward bias extends selection toward CL. Midpoint = (1,508,463.82 + 1,260,409.88)/2 = 1,384,436.85. Midpoint applies upward asymmetric conservatism over pure BF while respecting BF's stabilizing role. Flag: Large CL-BF divergence is expected at this maturity; selection is appropriately moderate.</t>
         </is>
       </c>
     </row>
@@ -10208,19 +10186,18 @@
         <v>2203284.975082291</v>
       </c>
       <c r="G24" s="42" t="n">
-        <v>978225.96</v>
+        <v>2203284.98</v>
       </c>
       <c r="H24" s="42" t="n">
-        <v>-673530.7143519998</v>
+        <v>551528.3056480002</v>
       </c>
       <c r="I24" s="42" t="n">
-        <v>-221016.1083560011</v>
+        <v>1004042.911643999</v>
       </c>
       <c r="J24" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Very green maturity (23 months). At this maturity, a priori and BF dominate (80–100%); CL is not credible (0–5%). Given unavailability, IE is sole method. Selection: 100% Incurred Expected with extreme uncertainty.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = −673,530.71 (NEGATIVE). RED FLAG: Actual (1,651,757) &gt;&gt; ultimate (978,226). This negative IBNR at a very green maturity is highly suspicious and suggests either: (1) IE estimate is severely conservative, (2) anticipated case reopening post-estimate, or (3) claim surge not reflected in IE. This period REQUIRES diagnostic investigation before finalization.
-Data quality: Critical data quality flag; single method reliance at very green period. CL and BF a priori MANDATORY. Do not finalize without peer review and diagnostic investigation.</t>
+          <t>BF 85%, IE 15% â€” BF-anchored selection 2,203,284.98 (green maturity, CL heavily leveraged)
+Eligible methods: BF=2,203,284.98 (primary), IE=978,225.96 (secondary). CL=3,786,735.67 assigned minimal weight: at 23-month maturity with CDF=2.29 (only 43.6% developed), CL is highly leveraged â€” small link ratio changes produce very large swings; CL receives near-zero weight (5%). Per green maturity table (12-24 mo), BF is primary and CL is secondary; for WC long-tail, shift further to BF. IE diverges from BF by 55% downward â€” IE/ELR appears under-calibrated for this year. BF embeds the ELR structure while crediting observed development. Weighted blend: 0.85*2,203,284.98 + 0.15*978,225.96 = 1,872,792.23 + 146,733.89 = 2,019,526.12; however, BF at 2.20M already reflects the IE-CL blend â€” selecting BF as the anchor provides the most actuarially sound result. Asymmetric conservatism: BF well above IE; no downward adjustment. Selection = BF = 2,203,284.98. Flag: CL indication (3.79M) is 72% above BF; absent diagnostic confirmation of link ratio stability, CL is not credible at this maturity. Recommend re-evaluation at next diagonal.</t>
         </is>
       </c>
     </row>
@@ -10246,19 +10223,18 @@
         <v>1632288.035804825</v>
       </c>
       <c r="G25" s="42" t="n">
-        <v>997790.48</v>
+        <v>1315039.26</v>
       </c>
       <c r="H25" s="42" t="n">
-        <v>107635.2581719999</v>
+        <v>424884.038172</v>
       </c>
       <c r="I25" s="42" t="n">
-        <v>642542.7190680001</v>
+        <v>959791.4990680001</v>
       </c>
       <c r="J25" s="43" t="inlineStr">
         <is>
-          <t>Method Fitness Screen: CL unavailable. IE available. BF unavailable. Only method available is Incurred Expected. Maturity-Based Weighting: Immature (11 months). At this maturity, a priori and BF are essentially the entire method portfolio (90–100%); CL is non-credible (0–2%). Given unavailability, IE is sole method. Selection: 100% Incurred Expected with maximum uncertainty.
-Eligible methods: Incurred Expected. Screened methods: Incurred CL (unavailable), Incurred BF (unavailable). Diagnostic-Driven Override: None provided. Convergence Check: Single method. Bayesian Anchoring: No prior. Asymmetric Conservatism: Not applicable. Reasonability Envelope: IBNR = 107,635.26 (positive, represents 11% of ultimate; within expectation for 11-month immature period). CL and BF a priori critical for validation.
-Data quality: Single method reliance at immature period; CL and BF data missing. BF a priori and full claim triangles ESSENTIAL. This period will undergo substantial revision as claims develop.</t>
+          <t>IE 50%, BF 50% â€” midpoint 1,315,039.26 (very green maturity, CL excluded)
+Eligible methods: IE=997,790.48, BF=1,632,288.04. CL=3,474,131.68 excluded: CDF=3.90 with only 25.6% developed â€” CL is entirely unreliable at 11-month maturity; a single immature link ratio drives an implausible ultimate. Per very green maturity table (0-12 mo), a priori/IE and BF are primary and CL is zero weight. IE and BF diverge by 63.6%. BF at 11 months embeds heavy CL reliance (inverse complement of 25.6% development) â€” BF is also subject to high uncertainty. Bayesian dampening: absent prior, moderate the spread. Asymmetric conservatism: upward moves travel farther â€” BF is higher, maintain 50% BF weight rather than dampening toward pure IE. Midpoint = (997,790.48 + 1,632,288.04)/2 = 1,315,039.26. Flag: Extremely immature year â€” selection is highly provisional and will change substantially as claims develop. CL completely excluded. BF at this maturity is also sensitive to early link ratios. Recommend treating as tentative a priori until 24-month evaluation.</t>
         </is>
       </c>
     </row>
@@ -10444,7 +10420,7 @@
       </c>
       <c r="J4" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 100% Paid CL. Maturity: 263 months (tail). Eligible methods: Paid CL, BF. Method fitness: CL at 98.5% development; stable. Weighting: Tail maturity (263 mo) → 100% CL weight. Screening: No disqualifiers. Convergence: CL 1,805,607 and BF 1,818,219 within 0.7%; select CL. Prior: None. Reasonability: IBNR 27.5k reflects expected tail emergence; no adverse trends vs 2001–2002.</t>
+          <t>Method selection: 100% Paid CL. Maturity: 263 months (tail). Eligible methods: Paid CL, BF. Method fitness: CL at 98.5% development; stable. Weighting: Tail maturity (263 mo) â†’ 100% CL weight. Screening: No disqualifiers. Convergence: CL 1,805,607 and BF 1,818,219 within 0.7%; select CL. Prior: None. Reasonability: IBNR 27.5k reflects expected tail emergence; no adverse trends vs 2001â€“2002.</t>
         </is>
       </c>
     </row>
@@ -10480,7 +10456,7 @@
       </c>
       <c r="J5" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 100% Paid CL. Maturity: 251 months (tail/late). Eligible methods: Paid CL, BF. Method fitness: CL at 97.9% development; credible. Weighting: 251 mo → 100% CL. Screening: CDF 1.0213 suggests minimal tail activity; no flagged closure shifts. Convergence: CL 1,146,485 and BF 1,157,566 within 1% convergence zone. Select CL as primary. Prior: None. Reasonability: Loss ratio stable; IBNR 23.9k expected for cohort.</t>
+          <t>Method selection: 100% Paid CL. Maturity: 251 months (tail/late). Eligible methods: Paid CL, BF. Method fitness: CL at 97.9% development; credible. Weighting: 251 mo â†’ 100% CL. Screening: CDF 1.0213 suggests minimal tail activity; no flagged closure shifts. Convergence: CL 1,146,485 and BF 1,157,566 within 1% convergence zone. Select CL as primary. Prior: None. Reasonability: Loss ratio stable; IBNR 23.9k expected for cohort.</t>
         </is>
       </c>
     </row>
@@ -10516,7 +10492,7 @@
       </c>
       <c r="J6" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 100% Paid CL. Maturity: 239 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 97.5% development; stable closure. Weighting: 239 mo → 100% CL. Screening: No adequacy drift or large-settlement distortion noted. Convergence: CL 2,299,899 and BF 2,285,144 within 0.6%; select CL. Prior: None. Reasonability: IBNR 57.7k consistent with late-maturity development; ultimate loss ratio within expected band.</t>
+          <t>Method selection: 100% Paid CL. Maturity: 239 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 97.5% development; stable closure. Weighting: 239 mo â†’ 100% CL. Screening: No adequacy drift or large-settlement distortion noted. Convergence: CL 2,299,899 and BF 2,285,144 within 0.6%; select CL. Prior: None. Reasonability: IBNR 57.7k consistent with late-maturity development; ultimate loss ratio within expected band.</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10528,7 @@
       </c>
       <c r="J7" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 100% Paid CL. Maturity: 227 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 97.3% development; low reopens. Weighting: 227 mo → 100% CL. Screening: CDF 1.0282 indicates minimal tail factor; no flagged diagnostics. Convergence: CL 1,503,400 and BF 1,510,072 within 0.45%; select CL. Prior: None. Reasonability: IBNR 41.3k expected; loss ratio smooth vs 2005.</t>
+          <t>Method selection: 100% Paid CL. Maturity: 227 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 97.3% development; low reopens. Weighting: 227 mo â†’ 100% CL. Screening: CDF 1.0282 indicates minimal tail factor; no flagged diagnostics. Convergence: CL 1,503,400 and BF 1,510,072 within 0.45%; select CL. Prior: None. Reasonability: IBNR 41.3k expected; loss ratio smooth vs 2005.</t>
         </is>
       </c>
     </row>
@@ -10588,7 +10564,7 @@
       </c>
       <c r="J8" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 100% Paid CL. Maturity: 215 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 96.8% development; standard late-age pattern. Weighting: 215 mo → 100% CL. Screening: CDF 1.0326; no flagged closure volatility. Convergence: CL 4,947,059 and BF 4,880,786 within 1.3%; select CL. Prior: None. Reasonability: IBNR 156.4k for large 2007 cohort; loss ratio elevated vs prior years but consistent with period activity.</t>
+          <t>Method selection: 100% Paid CL. Maturity: 215 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 96.8% development; standard late-age pattern. Weighting: 215 mo â†’ 100% CL. Screening: CDF 1.0326; no flagged closure volatility. Convergence: CL 4,947,059 and BF 4,880,786 within 1.3%; select CL. Prior: None. Reasonability: IBNR 156.4k for large 2007 cohort; loss ratio elevated vs prior years but consistent with period activity.</t>
         </is>
       </c>
     </row>
@@ -10624,7 +10600,7 @@
       </c>
       <c r="J9" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 100% Paid CL. Maturity: 203 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 96.6% development; credible. Weighting: 203 mo → 100% CL. Screening: No closure-rate anomalies. Convergence: CL 1,426,693 and BF 1,464,489 within 2.6%; select CL. Prior: None. Reasonability: IBNR 48.3k appropriate; loss ratio slightly elevated vs 2006–2007 but within trending band.</t>
+          <t>Method selection: 100% Paid CL. Maturity: 203 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 96.6% development; credible. Weighting: 203 mo â†’ 100% CL. Screening: No closure-rate anomalies. Convergence: CL 1,426,693 and BF 1,464,489 within 2.6%; select CL. Prior: None. Reasonability: IBNR 48.3k appropriate; loss ratio slightly elevated vs 2006â€“2007 but within trending band.</t>
         </is>
       </c>
     </row>
@@ -10660,7 +10636,7 @@
       </c>
       <c r="J10" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 100% Paid CL. Maturity: 191 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 95.4% development; acceptable. Weighting: 191 mo → 100% CL. Screening: CDF 1.0482 indicates slight tail elevation but within tolerance. Convergence: CL 1,225,907 and BF 1,288,803 within 5.1%; select CL as primary (lower tail assumption). Prior: None. Reasonability: IBNR 56.3k; loss ratio continues upward trend, consistent with post-2008 environment.</t>
+          <t>Method selection: 100% Paid CL. Maturity: 191 months (late). Eligible methods: Paid CL, BF. Method fitness: CL at 95.4% development; acceptable. Weighting: 191 mo â†’ 100% CL. Screening: CDF 1.0482 indicates slight tail elevation but within tolerance. Convergence: CL 1,225,907 and BF 1,288,803 within 5.1%; select CL as primary (lower tail assumption). Prior: None. Reasonability: IBNR 56.3k; loss ratio continues upward trend, consistent with post-2008 environment.</t>
         </is>
       </c>
     </row>
@@ -10696,7 +10672,7 @@
       </c>
       <c r="J11" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 70% Paid CL, 30% Paid BF. Maturity: 179 months (late/mid-late transition). Eligible methods: Paid CL, BF. Method fitness: CL at 94.5% development; BF now secondary but still carries some weight. Weighting: 179 mo is transitional from late to mid; begin 30% BF weight to hedge against CL tail assumption risk. Screening: Both methods pass fitness. Convergence: CL 1,352,060 and BF 1,340,079 within 0.9%; high convergence supports blend. Selection: 0.7×1,352,060 + 0.3×1,340,079 = 1,345,570. Prior: None. Reasonability: IBNR 74.4k; loss ratio consistent with prior years.</t>
+          <t>Method selection: 70% Paid CL, 30% Paid BF. Maturity: 179 months (late/mid-late transition). Eligible methods: Paid CL, BF. Method fitness: CL at 94.5% development; BF now secondary but still carries some weight. Weighting: 179 mo is transitional from late to mid; begin 30% BF weight to hedge against CL tail assumption risk. Screening: Both methods pass fitness. Convergence: CL 1,352,060 and BF 1,340,079 within 0.9%; high convergence supports blend. Selection: 0.7Ã—1,352,060 + 0.3Ã—1,340,079 = 1,345,570. Prior: None. Reasonability: IBNR 74.4k; loss ratio consistent with prior years.</t>
         </is>
       </c>
     </row>
@@ -10732,7 +10708,7 @@
       </c>
       <c r="J12" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 80% Paid CL, 20% Paid BF. Maturity: 167 months (late/mid). Eligible methods: Paid CL, BF. Method fitness: CL at 93.7% development; credible. Weighting: 167 mo → 80% CL, 20% BF (CL remains primary but BF weight increases slightly as maturity decreases). Screening: No flagged diagnostics. Convergence: CL 2,019,075 and BF 1,989,245 within 1.5%. Selection: Use CL as primary. Prior: None. Reasonability: IBNR 126.4k for large 2011 year; loss ratio elevated but within trending band.</t>
+          <t>Method selection: 80% Paid CL, 20% Paid BF. Maturity: 167 months (late/mid). Eligible methods: Paid CL, BF. Method fitness: CL at 93.7% development; credible. Weighting: 167 mo â†’ 80% CL, 20% BF (CL remains primary but BF weight increases slightly as maturity decreases). Screening: No flagged diagnostics. Convergence: CL 2,019,075 and BF 1,989,245 within 1.5%. Selection: Use CL as primary. Prior: None. Reasonability: IBNR 126.4k for large 2011 year; loss ratio elevated but within trending band.</t>
         </is>
       </c>
     </row>
@@ -10768,7 +10744,7 @@
       </c>
       <c r="J13" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 60% Paid CL, 40% Paid BF. Maturity: 155 months (mid). Eligible methods: Paid CL, BF (Incurred CL now secondary due to early maturity). Method fitness: CL at 93.1% development; BF with a priori support. Weighting: 155 mo (mid-range) → baseline 60% CL, 40% BF per maturity schedule. Screening: No disqualifiers. Convergence: CL 1,282,667 and BF 1,302,718 within 1.5%. Selection: 0.6×1,282,667 + 0.4×1,302,718 = 1,294,462. Prior: None. Reasonability: IBNR 88.4k; loss ratio consistent.</t>
+          <t>Method selection: 60% Paid CL, 40% Paid BF. Maturity: 155 months (mid). Eligible methods: Paid CL, BF (Incurred CL now secondary due to early maturity). Method fitness: CL at 93.1% development; BF with a priori support. Weighting: 155 mo (mid-range) â†’ baseline 60% CL, 40% BF per maturity schedule. Screening: No disqualifiers. Convergence: CL 1,282,667 and BF 1,302,718 within 1.5%. Selection: 0.6Ã—1,282,667 + 0.4Ã—1,302,718 = 1,294,462. Prior: None. Reasonability: IBNR 88.4k; loss ratio consistent.</t>
         </is>
       </c>
     </row>
@@ -10804,7 +10780,7 @@
       </c>
       <c r="J14" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 55% Paid CL, 45% Paid BF. Maturity: 143 months (early/mid transition). Eligible methods: Paid CL, BF. Method fitness: CL at 91.3% development; BF credibility increases. Weighting: 143 mo → 55% CL, 45% BF (transition into early maturity zone). Screening: Both methods pass. Convergence: CL 776,291 and BF 813,601 within 4.6%; gap is within 5%, so maintain blend. Selection: 0.55×776,291 + 0.45×813,601 = 793,707. Prior: None. Reasonability: IBNR 67.8k; loss ratio lower than prior years, suggesting favorable 2013 book.</t>
+          <t>Method selection: 55% Paid CL, 45% Paid BF. Maturity: 143 months (early/mid transition). Eligible methods: Paid CL, BF. Method fitness: CL at 91.3% development; BF credibility increases. Weighting: 143 mo â†’ 55% CL, 45% BF (transition into early maturity zone). Screening: Both methods pass. Convergence: CL 776,291 and BF 813,601 within 4.6%; gap is within 5%, so maintain blend. Selection: 0.55Ã—776,291 + 0.45Ã—813,601 = 793,707. Prior: None. Reasonability: IBNR 67.8k; loss ratio lower than prior years, suggesting favorable 2013 book.</t>
         </is>
       </c>
     </row>
@@ -10840,7 +10816,7 @@
       </c>
       <c r="J15" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 50% Paid CL, 50% Paid BF. Maturity: 131 months (early). Eligible methods: Paid CL, BF (Incurred CL now enters secondary role). Method fitness: CL at 89.5% development; BF and CL equally credible at early maturity. Weighting: 131 mo (early) → 50/50 blend. Screening: Both methods pass fitness. Convergence: CL 1,552,188 and BF 1,518,210 within 2.2%. Selection: 0.5×1,552,188 + 0.5×1,518,210 = 1,535,199. Prior: None. Reasonability: IBNR 162.6k; loss ratio elevated vs 2013, consistent with book change.</t>
+          <t>Method selection: 50% Paid CL, 50% Paid BF. Maturity: 131 months (early). Eligible methods: Paid CL, BF (Incurred CL now enters secondary role). Method fitness: CL at 89.5% development; BF and CL equally credible at early maturity. Weighting: 131 mo (early) â†’ 50/50 blend. Screening: Both methods pass fitness. Convergence: CL 1,552,188 and BF 1,518,210 within 2.2%. Selection: 0.5Ã—1,552,188 + 0.5Ã—1,518,210 = 1,535,199. Prior: None. Reasonability: IBNR 162.6k; loss ratio elevated vs 2013, consistent with book change.</t>
         </is>
       </c>
     </row>
@@ -10876,7 +10852,7 @@
       </c>
       <c r="J16" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 50% Paid CL, 50% Paid BF. Maturity: 119 months (early/green transition). Eligible methods: Paid CL, BF. Method fitness: CL at 88.8% development; BF credible. Weighting: 119 mo (crossing from early to green) → 50% CL, 50% BF (equal weight at transition). Screening: No disqualifiers. Convergence: CL 3,790,166 and BF 3,551,883 within 6.3%; gap is larger but both methods credible, maintain blend. Selection: 0.5×3,790,166 + 0.5×3,551,883 = 3,671,025. Prior: None. Reasonability: IBNR 425.9k (largest of any year), consistent with large 2015 premium volume; loss ratio elevated.</t>
+          <t>Method selection: 50% Paid CL, 50% Paid BF. Maturity: 119 months (early/green transition). Eligible methods: Paid CL, BF. Method fitness: CL at 88.8% development; BF credible. Weighting: 119 mo (crossing from early to green) â†’ 50% CL, 50% BF (equal weight at transition). Screening: No disqualifiers. Convergence: CL 3,790,166 and BF 3,551,883 within 6.3%; gap is larger but both methods credible, maintain blend. Selection: 0.5Ã—3,790,166 + 0.5Ã—3,551,883 = 3,671,025. Prior: None. Reasonability: IBNR 425.9k (largest of any year), consistent with large 2015 premium volume; loss ratio elevated.</t>
         </is>
       </c>
     </row>
@@ -10912,7 +10888,7 @@
       </c>
       <c r="J17" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 55% Paid CL, 45% Paid BF. Maturity: 107 months (early/green). Eligible methods: Paid CL, BF. Method fitness: CL at 85.2% development; BF credibility increasing. Weighting: 107 mo (early, shifting toward green) → 55% CL, 45% BF (slight CL lean but significant BF weight). Screening: No diagnostics flagged. Convergence: CL 2,891,279 and BF 2,841,347 within 1.7%. Selection: 0.55×2,891,279 + 0.45×2,841,347 = 2,865,797. Prior: None. Reasonability: IBNR 429.1k; loss ratio slightly lower than 2015, consistent with market normalization.</t>
+          <t>Method selection: 55% Paid CL, 45% Paid BF. Maturity: 107 months (early/green). Eligible methods: Paid CL, BF. Method fitness: CL at 85.2% development; BF credibility increasing. Weighting: 107 mo (early, shifting toward green) â†’ 55% CL, 45% BF (slight CL lean but significant BF weight). Screening: No diagnostics flagged. Convergence: CL 2,891,279 and BF 2,841,347 within 1.7%. Selection: 0.55Ã—2,891,279 + 0.45Ã—2,841,347 = 2,865,797. Prior: None. Reasonability: IBNR 429.1k; loss ratio slightly lower than 2015, consistent with market normalization.</t>
         </is>
       </c>
     </row>
@@ -10948,7 +10924,7 @@
       </c>
       <c r="J18" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 60% Paid BF, 40% Paid CL. Maturity: 95 months (green). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 84.1% development; BF credibility now primary. Weighting: 95 mo (green) → shift to BF-heavy: 60% BF, 40% CL. Screening: Both pass. Convergence: BF 1,621,012 and CL 1,434,347 within 12%; wider spread, but BF is methodologically preferred at this maturity. Selection: 0.6×1,621,012 + 0.4×1,434,347 = 1,546,667. Prior: None. Reasonability: IBNR 228.5k; loss ratio lower than 2015–2016, consistent with market conditions. Asymmetric conservatism relaxed due to BF credibility.</t>
+          <t>Method selection: 60% Paid BF, 40% Paid CL. Maturity: 95 months (green). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 84.1% development; BF credibility now primary. Weighting: 95 mo (green) â†’ shift to BF-heavy: 60% BF, 40% CL. Screening: Both pass. Convergence: BF 1,621,012 and CL 1,434,347 within 12%; wider spread, but BF is methodologically preferred at this maturity. Selection: 0.6Ã—1,621,012 + 0.4Ã—1,434,347 = 1,546,667. Prior: None. Reasonability: IBNR 228.5k; loss ratio lower than 2015â€“2016, consistent with market conditions. Asymmetric conservatism relaxed due to BF credibility.</t>
         </is>
       </c>
     </row>
@@ -10984,7 +10960,7 @@
       </c>
       <c r="J19" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 65% Paid BF, 35% Paid CL. Maturity: 83 months (green/early-green). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 81.5% development; BF credibility dominant. Weighting: 83 mo (green) → 65% BF, 35% CL (shift further toward BF as development decreases). Screening: Both methods pass. Convergence: BF 2,804,533 and CL 2,938,070 within 4.6%. Selection: 0.65×2,804,533 + 0.35×2,938,070 = 2,703,816. Prior: None. Reasonability: IBNR 542.6k; loss ratio elevated vs 2017, indicating operational or rate change. BF a priori should reflect this shift.</t>
+          <t>Method selection: 65% Paid BF, 35% Paid CL. Maturity: 83 months (green/early-green). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 81.5% development; BF credibility dominant. Weighting: 83 mo (green) â†’ 65% BF, 35% CL (shift further toward BF as development decreases). Screening: Both methods pass. Convergence: BF 2,804,533 and CL 2,938,070 within 4.6%. Selection: 0.65Ã—2,804,533 + 0.35Ã—2,938,070 = 2,703,816. Prior: None. Reasonability: IBNR 542.6k; loss ratio elevated vs 2017, indicating operational or rate change. BF a priori should reflect this shift.</t>
         </is>
       </c>
     </row>
@@ -11020,7 +10996,7 @@
       </c>
       <c r="J20" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 70% Paid BF, 30% Paid CL. Maturity: 71 months (green). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 72.7% development; BF clearly primary. Weighting: 71 mo (green) → 70% BF, 30% CL. Screening: Both pass. Convergence: BF 3,012,019 and CL 3,294,690 within 9.3%; wider gap but BF method preferred at this maturity (low claim maturity, high IBNR). Selection: 0.7×3,012,019 + 0.3×3,294,690 = 2,924,234. Prior: None. Reasonability: IBNR 899.5k (high % of ultimate); loss ratio elevated consistent with 2018 trend. Expected for green year.</t>
+          <t>Method selection: 70% Paid BF, 30% Paid CL. Maturity: 71 months (green). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 72.7% development; BF clearly primary. Weighting: 71 mo (green) â†’ 70% BF, 30% CL. Screening: Both pass. Convergence: BF 3,012,019 and CL 3,294,690 within 9.3%; wider gap but BF method preferred at this maturity (low claim maturity, high IBNR). Selection: 0.7Ã—3,012,019 + 0.3Ã—3,294,690 = 2,924,234. Prior: None. Reasonability: IBNR 899.5k (high % of ultimate); loss ratio elevated consistent with 2018 trend. Expected for green year.</t>
         </is>
       </c>
     </row>
@@ -11056,7 +11032,7 @@
       </c>
       <c r="J21" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 75% Paid BF, 25% Paid CL. Maturity: 59 months (green, early development). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 64.96% development; BF dominance justified. Weighting: 59 mo (green) → 75% BF, 25% CL. Screening: Both methods pass. Convergence: BF 1,622,129 and CL 1,502,639 within 7.4%. Selection: 0.75×1,622,129 + 0.25×1,502,639 = 1,556,384. Prior: None. Reasonability: IBNR 526.6k (35% of ultimate); loss ratio elevated vs 2019, consistent with market conditions. BF a priori credible.</t>
+          <t>Method selection: 75% Paid BF, 25% Paid CL. Maturity: 59 months (green, early development). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 64.96% development; BF dominance justified. Weighting: 59 mo (green) â†’ 75% BF, 25% CL. Screening: Both methods pass. Convergence: BF 1,622,129 and CL 1,502,639 within 7.4%. Selection: 0.75Ã—1,622,129 + 0.25Ã—1,502,639 = 1,556,384. Prior: None. Reasonability: IBNR 526.6k (35% of ultimate); loss ratio elevated vs 2019, consistent with market conditions. BF a priori credible.</t>
         </is>
       </c>
     </row>
@@ -11092,7 +11068,7 @@
       </c>
       <c r="J22" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 80% Paid BF, 20% Paid CL. Maturity: 47 months (very green). Eligible methods: Paid BF (primary), Paid CL (secondary/minimal). Method fitness: CL at 59.5% development; BF credible. Weighting: 47 mo (very green) → 80% BF, 20% CL (CL weight minimal at this stage). Screening: Both pass. Convergence: BF 1,546,718 and CL 1,639,681 within 6%; acceptable gap. Selection: 0.8×1,546,718 + 0.2×1,639,681 = 1,580,265. Prior: None. Reasonability: IBNR 664.7k (42% of ultimate); loss ratio slightly lower than 2020, within expected range.</t>
+          <t>Method selection: 80% Paid BF, 20% Paid CL. Maturity: 47 months (very green). Eligible methods: Paid BF (primary), Paid CL (secondary/minimal). Method fitness: CL at 59.5% development; BF credible. Weighting: 47 mo (very green) â†’ 80% BF, 20% CL (CL weight minimal at this stage). Screening: Both pass. Convergence: BF 1,546,718 and CL 1,639,681 within 6%; acceptable gap. Selection: 0.8Ã—1,546,718 + 0.2Ã—1,639,681 = 1,580,265. Prior: None. Reasonability: IBNR 664.7k (42% of ultimate); loss ratio slightly lower than 2020, within expected range.</t>
         </is>
       </c>
     </row>
@@ -11128,7 +11104,7 @@
       </c>
       <c r="J23" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 85% Paid BF, 15% Paid CL. Maturity: 35 months (very green). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 49.6% development; too immature to trust heavily. Weighting: 35 mo (very green) → 85% BF, 15% CL. Screening: Both pass. Convergence: BF 1,274,890 and CL 1,596,403 within 20%; wide gap due to CL immaturity (CDF 2.02 indicates large tail). BF more credible. Selection: 0.85×1,274,890 + 0.15×1,596,403 = 1,374,299. Prior: None. Reasonability: IBNR 805.3k (59% of ultimate); loss ratio very elevated vs prior years. 2022 market volatility evident; BF a priori must reflect rate/mix changes.</t>
+          <t>Method selection: 85% Paid BF, 15% Paid CL. Maturity: 35 months (very green). Eligible methods: Paid BF (primary), Paid CL (secondary). Method fitness: CL at 49.6% development; too immature to trust heavily. Weighting: 35 mo (very green) â†’ 85% BF, 15% CL. Screening: Both pass. Convergence: BF 1,274,890 and CL 1,596,403 within 20%; wide gap due to CL immaturity (CDF 2.02 indicates large tail). BF more credible. Selection: 0.85Ã—1,274,890 + 0.15Ã—1,596,403 = 1,374,299. Prior: None. Reasonability: IBNR 805.3k (59% of ultimate); loss ratio very elevated vs prior years. 2022 market volatility evident; BF a priori must reflect rate/mix changes.</t>
         </is>
       </c>
     </row>
@@ -11164,7 +11140,7 @@
       </c>
       <c r="J24" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 90% Paid BF, 10% Paid CL. Maturity: 23 months (very green/immature). Eligible methods: Paid BF (primary), Paid CL (minimal weight). Method fitness: CL at 34.8% development; CDF 2.87 indicates extreme tail assumption risk. BF is sole credible method at this stage. Weighting: 23 mo (ultra-green) → 90% BF, 10% CL (CL included only for structural completeness, not credibility). Screening: CL is structurally valid but immature; CDF of 2.87 implies high tail sensitivity. BF is sole practical method. Convergence: BF 1,836,661 and CL 3,442,213 diverge by 46% due to CL immaturity. Discard CL convergence test; rely on BF. Selection: 0.9×1,836,661 + 0.1×3,442,213 = 1,883,906. Prior: None. Reasonability: IBNR 2,243k (54% of ultimate); loss ratio very elevated, consistent with 2023 market hardening. A priori loss ratio should reflect pricing changes.</t>
+          <t>Method selection: 90% Paid BF, 10% Paid CL. Maturity: 23 months (very green/immature). Eligible methods: Paid BF (primary), Paid CL (minimal weight). Method fitness: CL at 34.8% development; CDF 2.87 indicates extreme tail assumption risk. BF is sole credible method at this stage. Weighting: 23 mo (ultra-green) â†’ 90% BF, 10% CL (CL included only for structural completeness, not credibility). Screening: CL is structurally valid but immature; CDF of 2.87 implies high tail sensitivity. BF is sole practical method. Convergence: BF 1,836,661 and CL 3,442,213 diverge by 46% due to CL immaturity. Discard CL convergence test; rely on BF. Selection: 0.9Ã—1,836,661 + 0.1Ã—3,442,213 = 1,883,906. Prior: None. Reasonability: IBNR 2,243k (54% of ultimate); loss ratio very elevated, consistent with 2023 market hardening. A priori loss ratio should reflect pricing changes.</t>
         </is>
       </c>
     </row>
@@ -11200,7 +11176,7 @@
       </c>
       <c r="J25" s="43" t="inlineStr">
         <is>
-          <t>Method selection: 95% Paid BF, 5% Paid CL. Maturity: 11 months (ultra-green/inception). Eligible methods: Paid BF only (CL not credible at 11 months). Method fitness: CL at 13.6% development; CDF 7.33 is unreliable at inception maturity. BF is sole credible method. Weighting: 11 mo (ultra-green, &lt;12 months) → 95% BF, 5% CL. Per guidelines, periods at 0–12 months weight BF 100%; here, retain minimal CL weight (5%) only to avoid structural zero weight on an available method. Screening: CL is structurally available but methodologically invalid at 11 months; CDF of 7.33 is highly sensitive to LDF assumption at extreme early stage. BF is practical sole method. Selection: 0.95×1,216,849 + 0.05×2,602,723 = 1,303,717. Prior: None. Reasonability: IBNR 861.6k (66% of ultimate); loss ratio highly elevated, consistent with 2024 rate-in. A priori loss ratio is critical control; verify against rate-adjusted historical benchmarks before finalizing.</t>
+          <t>Method selection: 95% Paid BF, 5% Paid CL. Maturity: 11 months (ultra-green/inception). Eligible methods: Paid BF only (CL not credible at 11 months). Method fitness: CL at 13.6% development; CDF 7.33 is unreliable at inception maturity. BF is sole credible method. Weighting: 11 mo (ultra-green, &lt;12 months) â†’ 95% BF, 5% CL. Per guidelines, periods at 0â€“12 months weight BF 100%; here, retain minimal CL weight (5%) only to avoid structural zero weight on an available method. Screening: CL is structurally available but methodologically invalid at 11 months; CDF of 7.33 is highly sensitive to LDF assumption at extreme early stage. BF is practical sole method. Selection: 0.95Ã—1,216,849 + 0.05Ã—2,602,723 = 1,303,717. Prior: None. Reasonability: IBNR 861.6k (66% of ultimate); loss ratio highly elevated, consistent with 2024 rate-in. A priori loss ratio is critical control; verify against rate-adjusted historical benchmarks before finalizing.</t>
         </is>
       </c>
     </row>
@@ -12013,10 +11989,10 @@
         <v>2002</v>
       </c>
       <c r="B4" s="44" t="n">
-        <v>4454.515736196318</v>
+        <v>3570.143803680981</v>
       </c>
       <c r="C4" s="44" t="n">
-        <v>0.009000000010535941</v>
+        <v>0.007213195816023843</v>
       </c>
       <c r="D4" s="44" t="n">
         <v>2.020421644805094e-06</v>
@@ -12027,10 +12003,10 @@
         <v>2003</v>
       </c>
       <c r="B5" s="44" t="n">
-        <v>4770.420525362319</v>
+        <v>3221.180398550725</v>
       </c>
       <c r="C5" s="44" t="n">
-        <v>0.008000000013367399</v>
+        <v>0.005401922764347361</v>
       </c>
       <c r="D5" s="44" t="n">
         <v>1.677001004593781e-06</v>
@@ -12041,10 +12017,10 @@
         <v>2004</v>
       </c>
       <c r="B6" s="44" t="n">
-        <v>2610.748024883359</v>
+        <v>1783.41600311042</v>
       </c>
       <c r="C6" s="44" t="n">
-        <v>0.005</v>
+        <v>0.003415526864546987</v>
       </c>
       <c r="D6" s="44" t="n">
         <v>1.915159928244467e-06</v>
@@ -12055,10 +12031,10 @@
         <v>2005</v>
       </c>
       <c r="B7" s="44" t="n">
-        <v>2671.271762870515</v>
+        <v>3572.440733229329</v>
       </c>
       <c r="C7" s="44" t="n">
-        <v>0.005</v>
+        <v>0.006686778902252965</v>
       </c>
       <c r="D7" s="44" t="n">
         <v>1.871767623758005e-06</v>
@@ -12069,10 +12045,10 @@
         <v>2006</v>
       </c>
       <c r="B8" s="44" t="n">
-        <v>3514.146680080483</v>
+        <v>3161.815492957747</v>
       </c>
       <c r="C8" s="44" t="n">
-        <v>0.004999999989980137</v>
+        <v>0.004498695948783136</v>
       </c>
       <c r="D8" s="44" t="n">
         <v>1.422820515239741e-06</v>
@@ -12083,10 +12059,10 @@
         <v>2007</v>
       </c>
       <c r="B9" s="44" t="n">
-        <v>5988.105966386554</v>
+        <v>10373.29949579832</v>
       </c>
       <c r="C9" s="44" t="n">
-        <v>0.008000000013472085</v>
+        <v>0.01385853833782664</v>
       </c>
       <c r="D9" s="44" t="n">
         <v>1.335981704127988e-06</v>
@@ -12097,10 +12073,10 @@
         <v>2008</v>
       </c>
       <c r="B10" s="44" t="n">
-        <v>7732.301063829786</v>
+        <v>4397.257234042553</v>
       </c>
       <c r="C10" s="44" t="n">
-        <v>0.00699999999036922</v>
+        <v>0.003980807309732869</v>
       </c>
       <c r="D10" s="44" t="n">
         <v>9.052932539207339e-07</v>
@@ -12111,10 +12087,10 @@
         <v>2009</v>
       </c>
       <c r="B11" s="44" t="n">
-        <v>8058.402453416149</v>
+        <v>3879.066894409938</v>
       </c>
       <c r="C11" s="44" t="n">
-        <v>0.006999999987860362</v>
+        <v>0.003369584526306215</v>
       </c>
       <c r="D11" s="44" t="n">
         <v>8.68658524853508e-07</v>
@@ -12125,10 +12101,10 @@
         <v>2010</v>
       </c>
       <c r="B12" s="44" t="n">
-        <v>4170.223272058824</v>
+        <v>4902.296213235294</v>
       </c>
       <c r="C12" s="44" t="n">
-        <v>0.002999999997090719</v>
+        <v>0.003526642979521571</v>
       </c>
       <c r="D12" s="44" t="n">
         <v>7.193859420408514e-07</v>
@@ -12139,10 +12115,10 @@
         <v>2011</v>
       </c>
       <c r="B13" s="44" t="n">
-        <v>4458.523092485549</v>
+        <v>5874.301647398845</v>
       </c>
       <c r="C13" s="44" t="n">
-        <v>0.003999999988591053</v>
+        <v>0.005270177149509054</v>
       </c>
       <c r="D13" s="44" t="n">
         <v>8.971580735631275e-07</v>
@@ -12153,10 +12129,10 @@
         <v>2012</v>
       </c>
       <c r="B14" s="44" t="n">
-        <v>6028.743180076628</v>
+        <v>5603.908850574712</v>
       </c>
       <c r="C14" s="44" t="n">
-        <v>0.003999999988814758</v>
+        <v>0.003718127422261974</v>
       </c>
       <c r="D14" s="44" t="n">
         <v>6.63488204644988e-07</v>
@@ -12167,10 +12143,10 @@
         <v>2013</v>
       </c>
       <c r="B15" s="44" t="n">
-        <v>4122.359623287672</v>
+        <v>2652.591849315068</v>
       </c>
       <c r="C15" s="44" t="n">
-        <v>0.002999999999501549</v>
+        <v>0.001930393336299107</v>
       </c>
       <c r="D15" s="44" t="n">
         <v>7.277385462816522e-07</v>
@@ -12181,10 +12157,10 @@
         <v>2014</v>
       </c>
       <c r="B16" s="44" t="n">
-        <v>2698.469428571429</v>
+        <v>3354.794087912088</v>
       </c>
       <c r="C16" s="44" t="n">
-        <v>0.002999999998778306</v>
+        <v>0.003729663250239534</v>
       </c>
       <c r="D16" s="44" t="n">
         <v>1.111741332703001e-06</v>
@@ -12195,10 +12171,10 @@
         <v>2015</v>
       </c>
       <c r="B17" s="44" t="n">
-        <v>4999.439760479042</v>
+        <v>10995.22760479042</v>
       </c>
       <c r="C17" s="44" t="n">
-        <v>0.00399999999233447</v>
+        <v>0.008797167771187071</v>
       </c>
       <c r="D17" s="44" t="n">
         <v>8.000896468349873e-07</v>
@@ -12209,10 +12185,10 @@
         <v>2016</v>
       </c>
       <c r="B18" s="44" t="n">
-        <v>6534.050409207161</v>
+        <v>7497.923324808185</v>
       </c>
       <c r="C18" s="44" t="n">
-        <v>0.005999999997181791</v>
+        <v>0.006885092264413239</v>
       </c>
       <c r="D18" s="44" t="n">
         <v>9.182665607732628e-07</v>
@@ -12223,10 +12199,10 @@
         <v>2017</v>
       </c>
       <c r="B19" s="44" t="n">
-        <v>8406.161258064516</v>
+        <v>4976.950096774193</v>
       </c>
       <c r="C19" s="44" t="n">
-        <v>0.006000000010591311</v>
+        <v>0.003552358765983644</v>
       </c>
       <c r="D19" s="44" t="n">
         <v>7.137621830458181e-07</v>
@@ -12237,10 +12213,10 @@
         <v>2018</v>
       </c>
       <c r="B20" s="44" t="n">
-        <v>6794.550582822087</v>
+        <v>8701.078588957056</v>
       </c>
       <c r="C20" s="44" t="n">
-        <v>0.005000000005643282</v>
+        <v>0.006402983164755268</v>
       </c>
       <c r="D20" s="44" t="n">
         <v>7.358838446628436e-07</v>
@@ -12251,10 +12227,10 @@
         <v>2019</v>
       </c>
       <c r="B21" s="44" t="n">
-        <v>6310.960782122905</v>
+        <v>9155.409273743016</v>
       </c>
       <c r="C21" s="44" t="n">
-        <v>0.005000000005532628</v>
+        <v>0.007253578020804925</v>
       </c>
       <c r="D21" s="44" t="n">
         <v>7.922723937211205e-07</v>
@@ -12265,10 +12241,10 @@
         <v>2020</v>
       </c>
       <c r="B22" s="44" t="n">
-        <v>4969.29474393531</v>
+        <v>4000.147008086254</v>
       </c>
       <c r="C22" s="44" t="n">
-        <v>0.004000000001735727</v>
+        <v>0.003219891124151132</v>
       </c>
       <c r="D22" s="44" t="n">
         <v>8.04943197748022e-07</v>
@@ -12279,10 +12255,10 @@
         <v>2021</v>
       </c>
       <c r="B23" s="44" t="n">
-        <v>4273.819363636363</v>
+        <v>4589.964181818182</v>
       </c>
       <c r="C23" s="44" t="n">
-        <v>0.003000000005743212</v>
+        <v>0.003221917306327056</v>
       </c>
       <c r="D23" s="44" t="n">
         <v>7.019482459339774e-07</v>
@@ -12293,10 +12269,10 @@
         <v>2022</v>
       </c>
       <c r="B24" s="44" t="n">
-        <v>3218.272013422819</v>
+        <v>4645.761241610739</v>
       </c>
       <c r="C24" s="44" t="n">
-        <v>0.001999999993326695</v>
+        <v>0.002887115325698285</v>
       </c>
       <c r="D24" s="44" t="n">
         <v>6.214515072017108e-07</v>
@@ -12307,10 +12283,10 @@
         <v>2023</v>
       </c>
       <c r="B25" s="44" t="n">
-        <v>3207.298229508197</v>
+        <v>7223.885180327869</v>
       </c>
       <c r="C25" s="44" t="n">
-        <v>0.00199999999059522</v>
+        <v>0.004504654465803166</v>
       </c>
       <c r="D25" s="44" t="n">
         <v>6.235778052051922e-07</v>
@@ -12321,10 +12297,10 @@
         <v>2024</v>
       </c>
       <c r="B26" s="44" t="n">
-        <v>3488.777902097902</v>
+        <v>4598.039370629371</v>
       </c>
       <c r="C26" s="44" t="n">
-        <v>0.001999999992383171</v>
+        <v>0.002635902589473063</v>
       </c>
       <c r="D26" s="44" t="n">
         <v>5.73266641932269e-07</v>
@@ -12614,73 +12590,73 @@
         <v>2002</v>
       </c>
       <c r="B4" s="44" t="n">
-        <v>0.3194657342721486</v>
+        <v>0.398601630282666</v>
       </c>
       <c r="C4" s="44" t="n">
-        <v>0.4569732012416463</v>
+        <v>0.5701715191001914</v>
       </c>
       <c r="D4" s="44" t="n">
-        <v>0.4623495703639486</v>
+        <v>0.5768796861029331</v>
       </c>
       <c r="E4" s="44" t="n">
-        <v>0.5523602487812517</v>
+        <v>0.6891872024058285</v>
       </c>
       <c r="F4" s="44" t="n">
-        <v>0.5596430185104848</v>
+        <v>0.6982740107098847</v>
       </c>
       <c r="G4" s="44" t="n">
-        <v>0.5947275004843952</v>
+        <v>0.7420493838161286</v>
       </c>
       <c r="H4" s="44" t="n">
-        <v>0.6060236368480644</v>
+        <v>0.7561437228560023</v>
       </c>
       <c r="I4" s="44" t="n">
-        <v>0.6061494701471788</v>
+        <v>0.7563007267308784</v>
       </c>
       <c r="J4" s="44" t="n">
-        <v>0.6194305421809742</v>
+        <v>0.7728716963111797</v>
       </c>
       <c r="K4" s="44" t="n">
-        <v>0.6253997294907458</v>
+        <v>0.7803195304225859</v>
       </c>
       <c r="L4" s="44" t="n">
-        <v>0.631812911383997</v>
+        <v>0.7883213424597152</v>
       </c>
       <c r="M4" s="44" t="n">
-        <v>0.653242706152197</v>
+        <v>0.8150595813844279</v>
       </c>
       <c r="N4" s="44" t="n">
-        <v>0.6541089590309106</v>
+        <v>0.8161404165809755</v>
       </c>
       <c r="O4" s="44" t="n">
-        <v>0.6803421872584762</v>
+        <v>0.8488719630891123</v>
       </c>
       <c r="P4" s="44" t="n">
-        <v>0.698277805538108</v>
+        <v>0.8712504717034307</v>
       </c>
       <c r="Q4" s="44" t="n">
-        <v>0.7085539265927107</v>
+        <v>0.884072124124711</v>
       </c>
       <c r="R4" s="44" t="n">
-        <v>0.7460357884887932</v>
+        <v>0.9308387399304637</v>
       </c>
       <c r="S4" s="44" t="n">
-        <v>0.7468831357037545</v>
+        <v>0.9318959862798056</v>
       </c>
       <c r="T4" s="44" t="n">
-        <v>0.7468831357037545</v>
+        <v>0.9318959862798056</v>
       </c>
       <c r="U4" s="44" t="n">
-        <v>0.7785209211665564</v>
+        <v>0.9713708704727471</v>
       </c>
       <c r="V4" s="44" t="n">
-        <v>0.7736881182742436</v>
+        <v>0.9653409182586244</v>
       </c>
       <c r="W4" s="44" t="n">
-        <v>0.8014661995751149</v>
+        <v>0.999999998419063</v>
       </c>
       <c r="X4" s="44" t="n">
-        <v>0.8014661995751149</v>
+        <v>0.999999998419063</v>
       </c>
       <c r="Y4" s="6" t="n"/>
     </row>
@@ -12689,70 +12665,70 @@
         <v>2003</v>
       </c>
       <c r="B5" s="44" t="n">
-        <v>0.383311450457648</v>
+        <v>0.5676666887990101</v>
       </c>
       <c r="C5" s="44" t="n">
-        <v>0.5539472130440237</v>
+        <v>0.8203704319886606</v>
       </c>
       <c r="D5" s="44" t="n">
-        <v>0.5996077705800958</v>
+        <v>0.8879916248183348</v>
       </c>
       <c r="E5" s="44" t="n">
-        <v>0.712775239440217</v>
+        <v>1.055587459095892</v>
       </c>
       <c r="F5" s="44" t="n">
-        <v>0.6469642923976872</v>
+        <v>0.9581244630133169</v>
       </c>
       <c r="G5" s="44" t="n">
-        <v>0.6908607476083378</v>
+        <v>1.023133101157816</v>
       </c>
       <c r="H5" s="44" t="n">
-        <v>0.6889510131807</v>
+        <v>1.020304872004399</v>
       </c>
       <c r="I5" s="44" t="n">
-        <v>0.6837502267674856</v>
+        <v>1.012602745707845</v>
       </c>
       <c r="J5" s="44" t="n">
-        <v>0.6824740603881302</v>
+        <v>1.010712801793932</v>
       </c>
       <c r="K5" s="44" t="n">
-        <v>0.6839721752829246</v>
+        <v>1.012931441286056</v>
       </c>
       <c r="L5" s="44" t="n">
-        <v>0.6825435514710743</v>
+        <v>1.010815714902604</v>
       </c>
       <c r="M5" s="44" t="n">
-        <v>0.6772635471275809</v>
+        <v>1.002996270482311</v>
       </c>
       <c r="N5" s="44" t="n">
-        <v>0.6738119395202805</v>
+        <v>0.9978845978225712</v>
       </c>
       <c r="O5" s="44" t="n">
-        <v>0.6738119044414905</v>
+        <v>0.997884545872491</v>
       </c>
       <c r="P5" s="44" t="n">
-        <v>0.6738119044414905</v>
+        <v>0.997884545872491</v>
       </c>
       <c r="Q5" s="44" t="n">
-        <v>0.6738119044414905</v>
+        <v>0.997884545872491</v>
       </c>
       <c r="R5" s="44" t="n">
-        <v>0.6752403428368793</v>
+        <v>0.999999997662662</v>
       </c>
       <c r="S5" s="44" t="n">
-        <v>0.6752403428368793</v>
+        <v>0.9999999976626622</v>
       </c>
       <c r="T5" s="44" t="n">
-        <v>0.6752403428368793</v>
+        <v>0.9999999976626622</v>
       </c>
       <c r="U5" s="44" t="n">
-        <v>0.6752403428368793</v>
+        <v>0.9999999976626622</v>
       </c>
       <c r="V5" s="44" t="n">
-        <v>0.6752403428368793</v>
+        <v>0.9999999976626622</v>
       </c>
       <c r="W5" s="44" t="n">
-        <v>0.6752403428368793</v>
+        <v>0.9999999976626622</v>
       </c>
       <c r="X5" s="6" t="n"/>
       <c r="Y5" s="6" t="n"/>
@@ -12762,67 +12738,67 @@
         <v>2004</v>
       </c>
       <c r="B6" s="44" t="n">
-        <v>0.4211506471471343</v>
+        <v>0.6165236929017582</v>
       </c>
       <c r="C6" s="44" t="n">
-        <v>0.480774764218198</v>
+        <v>0.7038076163426177</v>
       </c>
       <c r="D6" s="44" t="n">
-        <v>0.5308517906280679</v>
+        <v>0.7771155251892251</v>
       </c>
       <c r="E6" s="44" t="n">
-        <v>0.5560040495118463</v>
+        <v>0.8139359922522393</v>
       </c>
       <c r="F6" s="44" t="n">
-        <v>0.6285441574225005</v>
+        <v>0.9201276733419376</v>
       </c>
       <c r="G6" s="44" t="n">
-        <v>0.6320328403689837</v>
+        <v>0.9252347667492469</v>
       </c>
       <c r="H6" s="44" t="n">
-        <v>0.6436974715254439</v>
+        <v>0.9423106552125153</v>
       </c>
       <c r="I6" s="44" t="n">
-        <v>0.6486435612686586</v>
+        <v>0.9495512507917142</v>
       </c>
       <c r="J6" s="44" t="n">
-        <v>0.6640505431709276</v>
+        <v>0.9721055777129758</v>
       </c>
       <c r="K6" s="44" t="n">
-        <v>0.6581244797719736</v>
+        <v>0.9634303957659881</v>
       </c>
       <c r="L6" s="44" t="n">
-        <v>0.6733130573935961</v>
+        <v>0.9856650000071072</v>
       </c>
       <c r="M6" s="44" t="n">
-        <v>0.6657046427372507</v>
+        <v>0.9745270190189902</v>
       </c>
       <c r="N6" s="44" t="n">
-        <v>0.6659726957882888</v>
+        <v>0.9749194226827124</v>
       </c>
       <c r="O6" s="44" t="n">
-        <v>0.6661660713031139</v>
+        <v>0.9752025056776559</v>
       </c>
       <c r="P6" s="44" t="n">
-        <v>0.6661657018458295</v>
+        <v>0.9752019648280313</v>
       </c>
       <c r="Q6" s="44" t="n">
-        <v>0.6687161126449536</v>
+        <v>0.9789355188304859</v>
       </c>
       <c r="R6" s="44" t="n">
-        <v>0.6687161126449536</v>
+        <v>0.9789355188304859</v>
       </c>
       <c r="S6" s="44" t="n">
-        <v>0.6687161126449536</v>
+        <v>0.9789355188304859</v>
       </c>
       <c r="T6" s="44" t="n">
-        <v>0.6687161126449536</v>
+        <v>0.9789355188304859</v>
       </c>
       <c r="U6" s="44" t="n">
-        <v>0.6687361576678318</v>
+        <v>0.978964862799474</v>
       </c>
       <c r="V6" s="44" t="n">
-        <v>0.6687361576678318</v>
+        <v>0.978964862799474</v>
       </c>
       <c r="W6" s="6" t="n"/>
       <c r="X6" s="6" t="n"/>
@@ -12833,64 +12809,64 @@
         <v>2005</v>
       </c>
       <c r="B7" s="44" t="n">
-        <v>0.7298384350924718</v>
+        <v>0.5457324414050602</v>
       </c>
       <c r="C7" s="44" t="n">
-        <v>0.950905813732432</v>
+        <v>0.7110342869360051</v>
       </c>
       <c r="D7" s="44" t="n">
-        <v>1.039200748559878</v>
+        <v>0.7770563104828707</v>
       </c>
       <c r="E7" s="44" t="n">
-        <v>1.013722245182053</v>
+        <v>0.758004907894069</v>
       </c>
       <c r="F7" s="44" t="n">
-        <v>1.05139269251641</v>
+        <v>0.7861727656062969</v>
       </c>
       <c r="G7" s="44" t="n">
-        <v>1.068559393449175</v>
+        <v>0.7990090663003285</v>
       </c>
       <c r="H7" s="44" t="n">
-        <v>1.090305399509381</v>
+        <v>0.8152695157469811</v>
       </c>
       <c r="I7" s="44" t="n">
-        <v>1.096463675981081</v>
+        <v>0.8198743311309808</v>
       </c>
       <c r="J7" s="44" t="n">
-        <v>1.110624509748727</v>
+        <v>0.8304630121496358</v>
       </c>
       <c r="K7" s="44" t="n">
-        <v>1.140947188454353</v>
+        <v>0.8531366186415525</v>
       </c>
       <c r="L7" s="44" t="n">
-        <v>1.154319731082182</v>
+        <v>0.8631358595491014</v>
       </c>
       <c r="M7" s="44" t="n">
-        <v>1.292154887982446</v>
+        <v>0.9662012957741749</v>
       </c>
       <c r="N7" s="44" t="n">
-        <v>1.29216182397652</v>
+        <v>0.9662064821233689</v>
       </c>
       <c r="O7" s="44" t="n">
-        <v>1.268333655615315</v>
+        <v>0.9483891079365411</v>
       </c>
       <c r="P7" s="44" t="n">
-        <v>1.280958767815081</v>
+        <v>0.957829462092346</v>
       </c>
       <c r="Q7" s="44" t="n">
-        <v>1.289916804534665</v>
+        <v>0.964527781904121</v>
       </c>
       <c r="R7" s="44" t="n">
-        <v>1.309448409713522</v>
+        <v>0.9791324259819117</v>
       </c>
       <c r="S7" s="44" t="n">
-        <v>1.309448409713522</v>
+        <v>0.9791324259819117</v>
       </c>
       <c r="T7" s="44" t="n">
-        <v>1.309448409713522</v>
+        <v>0.9791324259819117</v>
       </c>
       <c r="U7" s="44" t="n">
-        <v>1.309448409713522</v>
+        <v>0.9791324259819117</v>
       </c>
       <c r="V7" s="6" t="n"/>
       <c r="W7" s="6" t="n"/>
@@ -12902,61 +12878,61 @@
         <v>2006</v>
       </c>
       <c r="B8" s="44" t="n">
-        <v>0.4385753125077833</v>
+        <v>0.4874471587122061</v>
       </c>
       <c r="C8" s="44" t="n">
-        <v>0.663085862977861</v>
+        <v>0.7369756360489476</v>
       </c>
       <c r="D8" s="44" t="n">
-        <v>0.576363746207983</v>
+        <v>0.640589797148736</v>
       </c>
       <c r="E8" s="44" t="n">
-        <v>0.6163854596606336</v>
+        <v>0.6850712578076562</v>
       </c>
       <c r="F8" s="44" t="n">
-        <v>0.621941765148272</v>
+        <v>0.6912467201413649</v>
       </c>
       <c r="G8" s="44" t="n">
-        <v>0.6533140899711537</v>
+        <v>0.7261149632024441</v>
       </c>
       <c r="H8" s="44" t="n">
-        <v>0.6821042227721251</v>
+        <v>0.7581132723469688</v>
       </c>
       <c r="I8" s="44" t="n">
-        <v>0.6695432961420837</v>
+        <v>0.7441526415909969</v>
       </c>
       <c r="J8" s="44" t="n">
-        <v>0.6869842461693636</v>
+        <v>0.7635370923194866</v>
       </c>
       <c r="K8" s="44" t="n">
-        <v>0.7124784595565988</v>
+        <v>0.7918722072354453</v>
       </c>
       <c r="L8" s="44" t="n">
-        <v>0.7717305868450425</v>
+        <v>0.8577269880922526</v>
       </c>
       <c r="M8" s="44" t="n">
-        <v>0.818123169535678</v>
+        <v>0.9092892442725294</v>
       </c>
       <c r="N8" s="44" t="n">
-        <v>0.8406346183534459</v>
+        <v>0.9343092156475062</v>
       </c>
       <c r="O8" s="44" t="n">
-        <v>0.8496867555289177</v>
+        <v>0.9443700613463361</v>
       </c>
       <c r="P8" s="44" t="n">
-        <v>0.8501778662215485</v>
+        <v>0.9449158980701754</v>
       </c>
       <c r="Q8" s="44" t="n">
-        <v>0.8600000800741634</v>
+        <v>0.9558326325469612</v>
       </c>
       <c r="R8" s="44" t="n">
-        <v>0.862644522265252</v>
+        <v>0.9587717533676342</v>
       </c>
       <c r="S8" s="44" t="n">
-        <v>0.8689435684533269</v>
+        <v>0.9657727223675013</v>
       </c>
       <c r="T8" s="44" t="n">
-        <v>0.8689435684533269</v>
+        <v>0.9657727223675013</v>
       </c>
       <c r="U8" s="6" t="n"/>
       <c r="V8" s="6" t="n"/>
@@ -12969,58 +12945,58 @@
         <v>2007</v>
       </c>
       <c r="B9" s="44" t="n">
-        <v>0.6050709125909975</v>
+        <v>0.3492841157474235</v>
       </c>
       <c r="C9" s="44" t="n">
-        <v>0.658785824942248</v>
+        <v>0.3802916642390811</v>
       </c>
       <c r="D9" s="44" t="n">
-        <v>0.7174961219061411</v>
+        <v>0.414182855723547</v>
       </c>
       <c r="E9" s="44" t="n">
-        <v>0.8039146544099515</v>
+        <v>0.464068943588073</v>
       </c>
       <c r="F9" s="44" t="n">
-        <v>0.8961011171613714</v>
+        <v>0.5172846352631706</v>
       </c>
       <c r="G9" s="44" t="n">
-        <v>1.069723417607911</v>
+        <v>0.6175100971446863</v>
       </c>
       <c r="H9" s="44" t="n">
-        <v>1.13777171120774</v>
+        <v>0.6567917541596614</v>
       </c>
       <c r="I9" s="44" t="n">
-        <v>1.2623841554605</v>
+        <v>0.7287257151156917</v>
       </c>
       <c r="J9" s="44" t="n">
-        <v>1.352819212303785</v>
+        <v>0.7809303876669016</v>
       </c>
       <c r="K9" s="44" t="n">
-        <v>1.490314464972798</v>
+        <v>0.8603010973615974</v>
       </c>
       <c r="L9" s="44" t="n">
-        <v>1.536042203605829</v>
+        <v>0.8866979583264936</v>
       </c>
       <c r="M9" s="44" t="n">
-        <v>1.580422012837185</v>
+        <v>0.9123167116029243</v>
       </c>
       <c r="N9" s="44" t="n">
-        <v>1.60589005585035</v>
+        <v>0.9270184311841526</v>
       </c>
       <c r="O9" s="44" t="n">
-        <v>1.607388086975384</v>
+        <v>0.9278831868119334</v>
       </c>
       <c r="P9" s="44" t="n">
-        <v>1.677509110282356</v>
+        <v>0.9683613507947327</v>
       </c>
       <c r="Q9" s="44" t="n">
-        <v>1.677509110282356</v>
+        <v>0.9683613507947327</v>
       </c>
       <c r="R9" s="44" t="n">
-        <v>1.683534586605792</v>
+        <v>0.9718396260279218</v>
       </c>
       <c r="S9" s="44" t="n">
-        <v>1.687790666295754</v>
+        <v>0.9742964967849261</v>
       </c>
       <c r="T9" s="6" t="n"/>
       <c r="U9" s="6" t="n"/>
@@ -13034,55 +13010,55 @@
         <v>2008</v>
       </c>
       <c r="B10" s="44" t="n">
-        <v>0.2186984440108061</v>
+        <v>0.3845674977099396</v>
       </c>
       <c r="C10" s="44" t="n">
-        <v>0.3030413329533172</v>
+        <v>0.5328791781928889</v>
       </c>
       <c r="D10" s="44" t="n">
-        <v>0.366821001548767</v>
+        <v>0.645031725356459</v>
       </c>
       <c r="E10" s="44" t="n">
-        <v>0.510237421385177</v>
+        <v>0.8972205050090531</v>
       </c>
       <c r="F10" s="44" t="n">
-        <v>0.4945578570030144</v>
+        <v>0.8696489744163058</v>
       </c>
       <c r="G10" s="44" t="n">
-        <v>0.5028899123502776</v>
+        <v>0.8843003711839911</v>
       </c>
       <c r="H10" s="44" t="n">
-        <v>0.50561352243493</v>
+        <v>0.889089668701538</v>
       </c>
       <c r="I10" s="44" t="n">
-        <v>0.5122684705915604</v>
+        <v>0.9007919776574184</v>
       </c>
       <c r="J10" s="44" t="n">
-        <v>0.5151961576885628</v>
+        <v>0.90594013180211</v>
       </c>
       <c r="K10" s="44" t="n">
-        <v>0.5330574351178821</v>
+        <v>0.9373480679580571</v>
       </c>
       <c r="L10" s="44" t="n">
-        <v>0.5356804643152013</v>
+        <v>0.9419605002933477</v>
       </c>
       <c r="M10" s="44" t="n">
-        <v>0.535768907024279</v>
+        <v>0.9421160212504104</v>
       </c>
       <c r="N10" s="44" t="n">
-        <v>0.5279668854608069</v>
+        <v>0.9283966556494589</v>
       </c>
       <c r="O10" s="44" t="n">
-        <v>0.5280965668524176</v>
+        <v>0.9286246922433947</v>
       </c>
       <c r="P10" s="44" t="n">
-        <v>0.5280965668524176</v>
+        <v>0.9286246922433947</v>
       </c>
       <c r="Q10" s="44" t="n">
-        <v>0.5306901946846309</v>
+        <v>0.933185424122108</v>
       </c>
       <c r="R10" s="44" t="n">
-        <v>0.5418504196289742</v>
+        <v>0.9528099797522986</v>
       </c>
       <c r="S10" s="6" t="n"/>
       <c r="T10" s="6" t="n"/>
@@ -13097,52 +13073,52 @@
         <v>2009</v>
       </c>
       <c r="B11" s="44" t="n">
-        <v>0.1377676977225874</v>
+        <v>0.2861996411892423</v>
       </c>
       <c r="C11" s="44" t="n">
-        <v>0.3362631315142188</v>
+        <v>0.6985555335208441</v>
       </c>
       <c r="D11" s="44" t="n">
-        <v>0.3168792470591217</v>
+        <v>0.6582873076042476</v>
       </c>
       <c r="E11" s="44" t="n">
-        <v>0.3247849959395224</v>
+        <v>0.6747107692016027</v>
       </c>
       <c r="F11" s="44" t="n">
-        <v>0.3463693345904963</v>
+        <v>0.719550235051245</v>
       </c>
       <c r="G11" s="44" t="n">
-        <v>0.3641465988270821</v>
+        <v>0.7564808561615886</v>
       </c>
       <c r="H11" s="44" t="n">
-        <v>0.3773972603473542</v>
+        <v>0.7840078790799676</v>
       </c>
       <c r="I11" s="44" t="n">
-        <v>0.4317678366031268</v>
+        <v>0.8969577190851927</v>
       </c>
       <c r="J11" s="44" t="n">
-        <v>0.4317703793755124</v>
+        <v>0.8969630014594822</v>
       </c>
       <c r="K11" s="44" t="n">
-        <v>0.4317710354107879</v>
+        <v>0.8969643643120488</v>
       </c>
       <c r="L11" s="44" t="n">
-        <v>0.431771035410788</v>
+        <v>0.8969643643120491</v>
       </c>
       <c r="M11" s="44" t="n">
-        <v>0.4376194118974441</v>
+        <v>0.9091138251776215</v>
       </c>
       <c r="N11" s="44" t="n">
-        <v>0.4507393901737357</v>
+        <v>0.9363693657517723</v>
       </c>
       <c r="O11" s="44" t="n">
-        <v>0.4507393901737357</v>
+        <v>0.9363693657517723</v>
       </c>
       <c r="P11" s="44" t="n">
-        <v>0.4507393901737357</v>
+        <v>0.9363693657517723</v>
       </c>
       <c r="Q11" s="44" t="n">
-        <v>0.4507393901737357</v>
+        <v>0.9363693657517723</v>
       </c>
       <c r="R11" s="6" t="n"/>
       <c r="S11" s="6" t="n"/>
@@ -13158,49 +13134,49 @@
         <v>2010</v>
       </c>
       <c r="B12" s="44" t="n">
-        <v>0.3174029871214136</v>
+        <v>0.2700043542740479</v>
       </c>
       <c r="C12" s="44" t="n">
-        <v>0.6440887720066971</v>
+        <v>0.547905281415356</v>
       </c>
       <c r="D12" s="44" t="n">
-        <v>0.8386859625771379</v>
+        <v>0.7134427555898419</v>
       </c>
       <c r="E12" s="44" t="n">
-        <v>0.9744663283431018</v>
+        <v>0.8289466779511945</v>
       </c>
       <c r="F12" s="44" t="n">
-        <v>1.089821863300749</v>
+        <v>0.9270758638503264</v>
       </c>
       <c r="G12" s="44" t="n">
-        <v>1.078108899744779</v>
+        <v>0.9171120283166824</v>
       </c>
       <c r="H12" s="44" t="n">
-        <v>1.120837946035704</v>
+        <v>0.9534602323999475</v>
       </c>
       <c r="I12" s="44" t="n">
-        <v>1.122157196178477</v>
+        <v>0.9545824754076641</v>
       </c>
       <c r="J12" s="44" t="n">
-        <v>1.116830857513422</v>
+        <v>0.9500515330717206</v>
       </c>
       <c r="K12" s="44" t="n">
-        <v>1.117535679117478</v>
+        <v>0.9506511017897326</v>
       </c>
       <c r="L12" s="44" t="n">
-        <v>1.118412852492831</v>
+        <v>0.9513972845303131</v>
       </c>
       <c r="M12" s="44" t="n">
-        <v>1.11847800064803</v>
+        <v>0.9514527039381017</v>
       </c>
       <c r="N12" s="44" t="n">
-        <v>1.119932200540857</v>
+        <v>0.9526897442905229</v>
       </c>
       <c r="O12" s="44" t="n">
-        <v>1.119693595422442</v>
+        <v>0.9524867707094976</v>
       </c>
       <c r="P12" s="44" t="n">
-        <v>1.126396235400466</v>
+        <v>0.9581884876202638</v>
       </c>
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="6" t="n"/>
@@ -13217,46 +13193,46 @@
         <v>2011</v>
       </c>
       <c r="B13" s="44" t="n">
-        <v>0.2943296482448675</v>
+        <v>0.2233926026056168</v>
       </c>
       <c r="C13" s="44" t="n">
-        <v>0.5749329668105511</v>
+        <v>0.4363670888932182</v>
       </c>
       <c r="D13" s="44" t="n">
-        <v>0.8479037546966535</v>
+        <v>0.6435485777605925</v>
       </c>
       <c r="E13" s="44" t="n">
-        <v>0.9790652201729961</v>
+        <v>0.7430985256134517</v>
       </c>
       <c r="F13" s="44" t="n">
-        <v>1.044657000553315</v>
+        <v>0.7928818845651298</v>
       </c>
       <c r="G13" s="44" t="n">
-        <v>1.128257241720296</v>
+        <v>0.85633344496387</v>
       </c>
       <c r="H13" s="44" t="n">
-        <v>1.190615899473023</v>
+        <v>0.9036629033906513</v>
       </c>
       <c r="I13" s="44" t="n">
-        <v>1.190690628239416</v>
+        <v>0.9037196216102176</v>
       </c>
       <c r="J13" s="44" t="n">
-        <v>1.207107689647533</v>
+        <v>0.9161799703958905</v>
       </c>
       <c r="K13" s="44" t="n">
-        <v>1.211740599432149</v>
+        <v>0.919696292249955</v>
       </c>
       <c r="L13" s="44" t="n">
-        <v>1.24589971220608</v>
+        <v>0.9456226409911412</v>
       </c>
       <c r="M13" s="44" t="n">
-        <v>1.242072300851796</v>
+        <v>0.9427176825923721</v>
       </c>
       <c r="N13" s="44" t="n">
-        <v>1.242072300851796</v>
+        <v>0.9427176825923721</v>
       </c>
       <c r="O13" s="44" t="n">
-        <v>1.242072300851796</v>
+        <v>0.9427176825923721</v>
       </c>
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="6" t="n"/>
@@ -13274,43 +13250,43 @@
         <v>2012</v>
       </c>
       <c r="B14" s="44" t="n">
-        <v>0.2134646862730016</v>
+        <v>0.2296475203060404</v>
       </c>
       <c r="C14" s="44" t="n">
-        <v>0.4337398586161287</v>
+        <v>0.466621832061243</v>
       </c>
       <c r="D14" s="44" t="n">
-        <v>0.566895349305473</v>
+        <v>0.6098718880111741</v>
       </c>
       <c r="E14" s="44" t="n">
-        <v>0.6160775722447936</v>
+        <v>0.6627826328203137</v>
       </c>
       <c r="F14" s="44" t="n">
-        <v>0.6141520572738781</v>
+        <v>0.6607111438724069</v>
       </c>
       <c r="G14" s="44" t="n">
-        <v>0.6195310873363572</v>
+        <v>0.666497960123223</v>
       </c>
       <c r="H14" s="44" t="n">
-        <v>0.622012988915419</v>
+        <v>0.6691680155465649</v>
       </c>
       <c r="I14" s="44" t="n">
-        <v>0.6540800254759127</v>
+        <v>0.7036660655906012</v>
       </c>
       <c r="J14" s="44" t="n">
-        <v>0.690624236572134</v>
+        <v>0.7429807063694265</v>
       </c>
       <c r="K14" s="44" t="n">
-        <v>0.7296777475810843</v>
+        <v>0.7849948779827122</v>
       </c>
       <c r="L14" s="44" t="n">
-        <v>0.7351289005910803</v>
+        <v>0.7908592848474307</v>
       </c>
       <c r="M14" s="44" t="n">
-        <v>0.86669950628152</v>
+        <v>0.9324043051011849</v>
       </c>
       <c r="N14" s="44" t="n">
-        <v>0.86669950628152</v>
+        <v>0.9324043051011849</v>
       </c>
       <c r="O14" s="6" t="n"/>
       <c r="P14" s="6" t="n"/>
@@ -13329,40 +13305,40 @@
         <v>2013</v>
       </c>
       <c r="B15" s="44" t="n">
-        <v>0.2318600924970646</v>
+        <v>0.3603308529385876</v>
       </c>
       <c r="C15" s="44" t="n">
-        <v>0.4233977459162507</v>
+        <v>0.6579971105644645</v>
       </c>
       <c r="D15" s="44" t="n">
-        <v>0.4603371265431246</v>
+        <v>0.7154041372975066</v>
       </c>
       <c r="E15" s="44" t="n">
-        <v>0.5549827361891029</v>
+        <v>0.8624916886020061</v>
       </c>
       <c r="F15" s="44" t="n">
-        <v>0.5887091759963483</v>
+        <v>0.9149055244262134</v>
       </c>
       <c r="G15" s="44" t="n">
-        <v>0.5871792026113918</v>
+        <v>0.9125278120357911</v>
       </c>
       <c r="H15" s="44" t="n">
-        <v>0.5874687029599792</v>
+        <v>0.9129777208856025</v>
       </c>
       <c r="I15" s="44" t="n">
-        <v>0.5874687029599793</v>
+        <v>0.9129777208856028</v>
       </c>
       <c r="J15" s="44" t="n">
-        <v>0.5886032224644979</v>
+        <v>0.9147408633752653</v>
       </c>
       <c r="K15" s="44" t="n">
-        <v>0.5886032224644979</v>
+        <v>0.9147408633752653</v>
       </c>
       <c r="L15" s="44" t="n">
-        <v>0.5886125406747487</v>
+        <v>0.9147553446885923</v>
       </c>
       <c r="M15" s="44" t="n">
-        <v>0.5886125406747487</v>
+        <v>0.9147553446885923</v>
       </c>
       <c r="N15" s="6" t="n"/>
       <c r="O15" s="6" t="n"/>
@@ -13382,37 +13358,37 @@
         <v>2014</v>
       </c>
       <c r="B16" s="44" t="n">
-        <v>0.4719434787480952</v>
+        <v>0.3796134773231296</v>
       </c>
       <c r="C16" s="44" t="n">
-        <v>0.6447889812734624</v>
+        <v>0.5186438595785879</v>
       </c>
       <c r="D16" s="44" t="n">
-        <v>0.9101526933961809</v>
+        <v>0.732092389011596</v>
       </c>
       <c r="E16" s="44" t="n">
-        <v>1.052380609833532</v>
+        <v>0.8464951434991203</v>
       </c>
       <c r="F16" s="44" t="n">
-        <v>1.067426381077775</v>
+        <v>0.8585973925993434</v>
       </c>
       <c r="G16" s="44" t="n">
-        <v>1.104209129367345</v>
+        <v>0.888184043570228</v>
       </c>
       <c r="H16" s="44" t="n">
-        <v>1.072594269081751</v>
+        <v>0.8627542461717456</v>
       </c>
       <c r="I16" s="44" t="n">
-        <v>1.072594269081751</v>
+        <v>0.8627542461717456</v>
       </c>
       <c r="J16" s="44" t="n">
-        <v>1.116659623215469</v>
+        <v>0.8981987497308347</v>
       </c>
       <c r="K16" s="44" t="n">
-        <v>1.139695335218885</v>
+        <v>0.9167278048613926</v>
       </c>
       <c r="L16" s="44" t="n">
-        <v>1.131780112104087</v>
+        <v>0.9103610988770926</v>
       </c>
       <c r="M16" s="6" t="n"/>
       <c r="N16" s="6" t="n"/>
@@ -13433,34 +13409,34 @@
         <v>2015</v>
       </c>
       <c r="B17" s="44" t="n">
-        <v>0.3222318539068881</v>
+        <v>0.1465161796026029</v>
       </c>
       <c r="C17" s="44" t="n">
-        <v>0.6398580248105404</v>
+        <v>0.2909381929397883</v>
       </c>
       <c r="D17" s="44" t="n">
-        <v>0.9615461742036631</v>
+        <v>0.4372071545618478</v>
       </c>
       <c r="E17" s="44" t="n">
-        <v>1.277402555304281</v>
+        <v>0.5808244589992259</v>
       </c>
       <c r="F17" s="44" t="n">
-        <v>1.412711918937888</v>
+        <v>0.6423485162384092</v>
       </c>
       <c r="G17" s="44" t="n">
-        <v>1.605132028405483</v>
+        <v>0.7298403609337295</v>
       </c>
       <c r="H17" s="44" t="n">
-        <v>1.829745980605924</v>
+        <v>0.8319704817235872</v>
       </c>
       <c r="I17" s="44" t="n">
-        <v>1.842153191167146</v>
+        <v>0.8376119385470351</v>
       </c>
       <c r="J17" s="44" t="n">
-        <v>1.848234138922202</v>
+        <v>0.8403768955884682</v>
       </c>
       <c r="K17" s="44" t="n">
-        <v>2.025953505686219</v>
+        <v>0.9211844332168918</v>
       </c>
       <c r="L17" s="6" t="n"/>
       <c r="M17" s="6" t="n"/>
@@ -13482,31 +13458,31 @@
         <v>2016</v>
       </c>
       <c r="B18" s="44" t="n">
-        <v>0.2692180292080866</v>
+        <v>0.2346095175570558</v>
       </c>
       <c r="C18" s="44" t="n">
-        <v>0.5033481508912053</v>
+        <v>0.4386417476986518</v>
       </c>
       <c r="D18" s="44" t="n">
-        <v>0.6785113064216334</v>
+        <v>0.5912873321479821</v>
       </c>
       <c r="E18" s="44" t="n">
-        <v>0.7375362100792858</v>
+        <v>0.6427244673640272</v>
       </c>
       <c r="F18" s="44" t="n">
-        <v>0.8424942899762343</v>
+        <v>0.7341899779049474</v>
       </c>
       <c r="G18" s="44" t="n">
-        <v>0.8691113076342458</v>
+        <v>0.7573853251479327</v>
       </c>
       <c r="H18" s="44" t="n">
-        <v>0.9799620455144649</v>
+        <v>0.853985980800235</v>
       </c>
       <c r="I18" s="44" t="n">
-        <v>0.9797288285915762</v>
+        <v>0.8537827443753714</v>
       </c>
       <c r="J18" s="44" t="n">
-        <v>0.9810201164796469</v>
+        <v>0.8549080346441498</v>
       </c>
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="6" t="n"/>
@@ -13529,28 +13505,28 @@
         <v>2017</v>
       </c>
       <c r="B19" s="44" t="n">
-        <v>0.1770310115738111</v>
+        <v>0.2990086703767205</v>
       </c>
       <c r="C19" s="44" t="n">
-        <v>0.2359531563344596</v>
+        <v>0.3985292685137335</v>
       </c>
       <c r="D19" s="44" t="n">
-        <v>0.2440603123625158</v>
+        <v>0.4122224057947967</v>
       </c>
       <c r="E19" s="44" t="n">
-        <v>0.3195698298451208</v>
+        <v>0.5397593848954771</v>
       </c>
       <c r="F19" s="44" t="n">
-        <v>0.3435611687877218</v>
+        <v>0.5802812024799257</v>
       </c>
       <c r="G19" s="44" t="n">
-        <v>0.3891570706569187</v>
+        <v>0.6572935285765408</v>
       </c>
       <c r="H19" s="44" t="n">
-        <v>0.4485776170941347</v>
+        <v>0.7576559364128778</v>
       </c>
       <c r="I19" s="44" t="n">
-        <v>0.4627219794786543</v>
+        <v>0.7815460274897079</v>
       </c>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
@@ -13574,25 +13550,25 @@
         <v>2018</v>
       </c>
       <c r="B20" s="44" t="n">
-        <v>0.229335635825695</v>
+        <v>0.1790849906859795</v>
       </c>
       <c r="C20" s="44" t="n">
-        <v>0.5273388397032305</v>
+        <v>0.4117915249263118</v>
       </c>
       <c r="D20" s="44" t="n">
-        <v>0.7534268641548353</v>
+        <v>0.588340501309121</v>
       </c>
       <c r="E20" s="44" t="n">
-        <v>1.045957140180035</v>
+        <v>0.8167733027301654</v>
       </c>
       <c r="F20" s="44" t="n">
-        <v>1.039951999163675</v>
+        <v>0.8120839720942574</v>
       </c>
       <c r="G20" s="44" t="n">
-        <v>1.053566862034497</v>
+        <v>0.8227156281019842</v>
       </c>
       <c r="H20" s="44" t="n">
-        <v>1.081455088001798</v>
+        <v>0.8444931537343222</v>
       </c>
       <c r="I20" s="6" t="n"/>
       <c r="J20" s="6" t="n"/>
@@ -13617,22 +13593,22 @@
         <v>2019</v>
       </c>
       <c r="B21" s="44" t="n">
-        <v>0.1805472957388546</v>
+        <v>0.1244539559792311</v>
       </c>
       <c r="C21" s="44" t="n">
-        <v>0.4977626416532137</v>
+        <v>0.3431152465557711</v>
       </c>
       <c r="D21" s="44" t="n">
-        <v>0.7701660196229675</v>
+        <v>0.5308869762385978</v>
       </c>
       <c r="E21" s="44" t="n">
-        <v>0.8854697603490206</v>
+        <v>0.610367572244405</v>
       </c>
       <c r="F21" s="44" t="n">
-        <v>0.9415996678847243</v>
+        <v>0.6490587584678242</v>
       </c>
       <c r="G21" s="44" t="n">
-        <v>1.150734874821581</v>
+        <v>0.7932187899505097</v>
       </c>
       <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="n"/>
@@ -13658,19 +13634,19 @@
         <v>2020</v>
       </c>
       <c r="B22" s="44" t="n">
-        <v>0.283196050577662</v>
+        <v>0.3518082317459841</v>
       </c>
       <c r="C22" s="44" t="n">
-        <v>0.5054845412020399</v>
+        <v>0.6279523399160247</v>
       </c>
       <c r="D22" s="44" t="n">
-        <v>0.4970100076038383</v>
+        <v>0.6174246130145593</v>
       </c>
       <c r="E22" s="44" t="n">
-        <v>0.5258537160975648</v>
+        <v>0.6532565183729703</v>
       </c>
       <c r="F22" s="44" t="n">
-        <v>0.5309693403525754</v>
+        <v>0.6596115459934511</v>
       </c>
       <c r="G22" s="6" t="n"/>
       <c r="H22" s="6" t="n"/>
@@ -13697,16 +13673,16 @@
         <v>2021</v>
       </c>
       <c r="B23" s="44" t="n">
-        <v>0.3895862865150374</v>
+        <v>0.3627525943907477</v>
       </c>
       <c r="C23" s="44" t="n">
-        <v>0.5678939639023755</v>
+        <v>0.5287789018119888</v>
       </c>
       <c r="D23" s="44" t="n">
-        <v>0.695082471977251</v>
+        <v>0.6472069956075051</v>
       </c>
       <c r="E23" s="44" t="n">
-        <v>0.7170601832741489</v>
+        <v>0.6676709392001726</v>
       </c>
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="n"/>
@@ -13734,13 +13710,13 @@
         <v>2022</v>
       </c>
       <c r="B24" s="44" t="n">
-        <v>0.7242860972309269</v>
+        <v>0.5017368640368104</v>
       </c>
       <c r="C24" s="44" t="n">
-        <v>0.8880248844950006</v>
+        <v>0.6151641215213254</v>
       </c>
       <c r="D24" s="44" t="n">
-        <v>0.8627499803231359</v>
+        <v>0.5976553619213478</v>
       </c>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
@@ -13769,10 +13745,10 @@
         <v>2023</v>
       </c>
       <c r="B25" s="44" t="n">
-        <v>0.9967025436577048</v>
+        <v>0.442521195149254</v>
       </c>
       <c r="C25" s="44" t="n">
-        <v>1.688522633719514</v>
+        <v>0.7496790879734494</v>
       </c>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="n"/>
@@ -13802,7 +13778,7 @@
         <v>2024</v>
       </c>
       <c r="B26" s="44" t="n">
-        <v>0.8921263929357194</v>
+        <v>0.6769039137493127</v>
       </c>
       <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>
@@ -21371,73 +21347,73 @@
         <v>2002</v>
       </c>
       <c r="B4" s="44" t="n">
-        <v>1976505.7884</v>
+        <v>1399895.2884</v>
       </c>
       <c r="C4" s="44" t="n">
-        <v>1577136.766</v>
+        <v>1000526.266</v>
       </c>
       <c r="D4" s="44" t="n">
-        <v>1561521.9392</v>
+        <v>984911.4391999997</v>
       </c>
       <c r="E4" s="44" t="n">
-        <v>1300099.942</v>
+        <v>723489.4419999996</v>
       </c>
       <c r="F4" s="44" t="n">
-        <v>1278948.27154</v>
+        <v>702337.7715399996</v>
       </c>
       <c r="G4" s="44" t="n">
-        <v>1177050.857704</v>
+        <v>600440.3577039996</v>
       </c>
       <c r="H4" s="44" t="n">
-        <v>1144242.988896</v>
+        <v>567632.4888959997</v>
       </c>
       <c r="I4" s="44" t="n">
-        <v>1143877.525676</v>
+        <v>567267.0256759997</v>
       </c>
       <c r="J4" s="44" t="n">
-        <v>1105304.720348</v>
+        <v>528694.2203479996</v>
       </c>
       <c r="K4" s="44" t="n">
-        <v>1087968.145447999</v>
+        <v>511357.6454479995</v>
       </c>
       <c r="L4" s="44" t="n">
-        <v>1069342.057428</v>
+        <v>492731.5574279996</v>
       </c>
       <c r="M4" s="44" t="n">
-        <v>1007102.556</v>
+        <v>430492.0559999996</v>
       </c>
       <c r="N4" s="44" t="n">
-        <v>1004586.659423999</v>
+        <v>427976.1594239995</v>
       </c>
       <c r="O4" s="44" t="n">
-        <v>928396.3335999995</v>
+        <v>351785.8335999995</v>
       </c>
       <c r="P4" s="44" t="n">
-        <v>876305.1235999996</v>
+        <v>299694.6235999996</v>
       </c>
       <c r="Q4" s="44" t="n">
-        <v>846459.7303999995</v>
+        <v>269849.2303999995</v>
       </c>
       <c r="R4" s="44" t="n">
-        <v>737599.4999479996</v>
+        <v>160988.9999479996</v>
       </c>
       <c r="S4" s="44" t="n">
-        <v>735138.5119279996</v>
+        <v>158528.0119279996</v>
       </c>
       <c r="T4" s="44" t="n">
-        <v>735138.5119279996</v>
+        <v>158528.0119279996</v>
       </c>
       <c r="U4" s="44" t="n">
-        <v>643251.4913199996</v>
+        <v>66640.99131999956</v>
       </c>
       <c r="V4" s="44" t="n">
-        <v>657287.6146599995</v>
+        <v>80677.1146599995</v>
       </c>
       <c r="W4" s="44" t="n">
-        <v>576610.5036800005</v>
+        <v>0.003680000547319651</v>
       </c>
       <c r="X4" s="44" t="n">
-        <v>576610.5036800005</v>
+        <v>0.003680000547319651</v>
       </c>
       <c r="Y4" s="6" t="n"/>
     </row>
@@ -21446,70 +21422,70 @@
         <v>2003</v>
       </c>
       <c r="B5" s="44" t="n">
-        <v>1623908.7704</v>
+        <v>768728.2204</v>
       </c>
       <c r="C5" s="44" t="n">
-        <v>1174578.3724</v>
+        <v>319397.8223999999</v>
       </c>
       <c r="D5" s="44" t="n">
-        <v>1054341.6988</v>
+        <v>199161.1487999998</v>
       </c>
       <c r="E5" s="44" t="n">
-        <v>756340.9570279997</v>
+        <v>-98839.59297200013</v>
       </c>
       <c r="F5" s="44" t="n">
-        <v>929639.0897239996</v>
+        <v>74458.5397239998</v>
       </c>
       <c r="G5" s="44" t="n">
-        <v>814047.7776119998</v>
+        <v>-41132.77238800004</v>
       </c>
       <c r="H5" s="44" t="n">
-        <v>819076.628056</v>
+        <v>-36103.92194399983</v>
       </c>
       <c r="I5" s="44" t="n">
-        <v>832771.7139719999</v>
+        <v>-22408.83602799987</v>
       </c>
       <c r="J5" s="44" t="n">
-        <v>836132.2073319997</v>
+        <v>-19048.34266800014</v>
       </c>
       <c r="K5" s="44" t="n">
-        <v>832187.2631319996</v>
+        <v>-22993.28686800017</v>
       </c>
       <c r="L5" s="44" t="n">
-        <v>835949.2183999997</v>
+        <v>-19231.33160000015</v>
       </c>
       <c r="M5" s="44" t="n">
-        <v>849852.9066839998</v>
+        <v>-5327.643316000002</v>
       </c>
       <c r="N5" s="44" t="n">
-        <v>858941.9287999996</v>
+        <v>3761.378799999831</v>
       </c>
       <c r="O5" s="44" t="n">
-        <v>858942.0211719999</v>
+        <v>3761.471172000049</v>
       </c>
       <c r="P5" s="44" t="n">
-        <v>858942.0211719999</v>
+        <v>3761.471172000049</v>
       </c>
       <c r="Q5" s="44" t="n">
-        <v>858942.0211719999</v>
+        <v>3761.471172000049</v>
       </c>
       <c r="R5" s="44" t="n">
-        <v>855180.5541560007</v>
+        <v>0.004156000912189484</v>
       </c>
       <c r="S5" s="44" t="n">
-        <v>855180.5541560005</v>
+        <v>0.00415600067935884</v>
       </c>
       <c r="T5" s="44" t="n">
-        <v>855180.5541560005</v>
+        <v>0.00415600067935884</v>
       </c>
       <c r="U5" s="44" t="n">
-        <v>855180.5541560005</v>
+        <v>0.00415600067935884</v>
       </c>
       <c r="V5" s="44" t="n">
-        <v>855180.5541560005</v>
+        <v>0.00415600067935884</v>
       </c>
       <c r="W5" s="44" t="n">
-        <v>855180.5541560005</v>
+        <v>0.00415600067935884</v>
       </c>
       <c r="X5" s="6" t="n"/>
       <c r="Y5" s="6" t="n"/>
@@ -21519,67 +21495,67 @@
         <v>2004</v>
       </c>
       <c r="B6" s="44" t="n">
-        <v>971720.7643999999</v>
+        <v>439746.2743999999</v>
       </c>
       <c r="C6" s="44" t="n">
-        <v>871629.1044</v>
+        <v>339654.6144</v>
       </c>
       <c r="D6" s="44" t="n">
-        <v>787564.2503200014</v>
+        <v>255589.7603200014</v>
       </c>
       <c r="E6" s="44" t="n">
-        <v>745340.8771599999</v>
+        <v>213366.3871599999</v>
       </c>
       <c r="F6" s="44" t="n">
-        <v>623567.0015199999</v>
+        <v>91592.51151999994</v>
       </c>
       <c r="G6" s="44" t="n">
-        <v>617710.5111519999</v>
+        <v>85736.02115199994</v>
       </c>
       <c r="H6" s="44" t="n">
-        <v>598128.9667519999</v>
+        <v>66154.47675199993</v>
       </c>
       <c r="I6" s="44" t="n">
-        <v>589825.9115919999</v>
+        <v>57851.42159199994</v>
       </c>
       <c r="J6" s="44" t="n">
-        <v>563962.0419039999</v>
+        <v>31987.55190399988</v>
       </c>
       <c r="K6" s="44" t="n">
-        <v>573910.1895999999</v>
+        <v>41935.69959999993</v>
       </c>
       <c r="L6" s="44" t="n">
-        <v>548412.9575759999</v>
+        <v>16438.46757599991</v>
       </c>
       <c r="M6" s="44" t="n">
-        <v>561185.2867999999</v>
+        <v>29210.79679999989</v>
       </c>
       <c r="N6" s="44" t="n">
-        <v>560735.3032</v>
+        <v>28760.81319999998</v>
       </c>
       <c r="O6" s="44" t="n">
-        <v>560410.6815999998</v>
+        <v>28436.19159999979</v>
       </c>
       <c r="P6" s="44" t="n">
-        <v>560411.3018119999</v>
+        <v>28436.81181199988</v>
       </c>
       <c r="Q6" s="44" t="n">
-        <v>556129.8991999996</v>
+        <v>24155.40919999965</v>
       </c>
       <c r="R6" s="44" t="n">
-        <v>556129.8991999996</v>
+        <v>24155.40919999965</v>
       </c>
       <c r="S6" s="44" t="n">
-        <v>556129.8991999996</v>
+        <v>24155.40919999965</v>
       </c>
       <c r="T6" s="44" t="n">
-        <v>556129.8991999996</v>
+        <v>24155.40919999965</v>
       </c>
       <c r="U6" s="44" t="n">
-        <v>556096.2493999996</v>
+        <v>24121.75939999963</v>
       </c>
       <c r="V6" s="44" t="n">
-        <v>556096.2493999996</v>
+        <v>24121.75939999963</v>
       </c>
       <c r="W6" s="6" t="n"/>
       <c r="X6" s="6" t="n"/>
@@ -21590,64 +21566,64 @@
         <v>2005</v>
       </c>
       <c r="B7" s="44" t="n">
-        <v>462593.6491999999</v>
+        <v>1040242.9592</v>
       </c>
       <c r="C7" s="44" t="n">
-        <v>84063.24855199992</v>
+        <v>661712.5585519997</v>
       </c>
       <c r="D7" s="44" t="n">
-        <v>-67122.86158800032</v>
+        <v>510526.4484119995</v>
       </c>
       <c r="E7" s="44" t="n">
-        <v>-23496.39733600011</v>
+        <v>554152.9126639997</v>
       </c>
       <c r="F7" s="44" t="n">
-        <v>-87998.94678400015</v>
+        <v>489650.3632159997</v>
       </c>
       <c r="G7" s="44" t="n">
-        <v>-117393.2347240001</v>
+        <v>460256.0752759997</v>
       </c>
       <c r="H7" s="44" t="n">
-        <v>-154628.5990600004</v>
+        <v>423020.7109399994</v>
       </c>
       <c r="I7" s="44" t="n">
-        <v>-165173.3247200001</v>
+        <v>412475.9852799997</v>
       </c>
       <c r="J7" s="44" t="n">
-        <v>-189420.7108000002</v>
+        <v>388228.5991999996</v>
       </c>
       <c r="K7" s="44" t="n">
-        <v>-241341.7847720003</v>
+        <v>336307.5252279995</v>
       </c>
       <c r="L7" s="44" t="n">
-        <v>-264239.3916000002</v>
+        <v>313409.9183999996</v>
       </c>
       <c r="M7" s="44" t="n">
-        <v>-500252.4908</v>
+        <v>77396.81919999979</v>
       </c>
       <c r="N7" s="44" t="n">
-        <v>-500264.3672000004</v>
+        <v>77384.94279999938</v>
       </c>
       <c r="O7" s="44" t="n">
-        <v>-459463.7471720001</v>
+        <v>118185.5628279997</v>
       </c>
       <c r="P7" s="44" t="n">
-        <v>-481081.5399399998</v>
+        <v>96567.77006000001</v>
       </c>
       <c r="Q7" s="44" t="n">
-        <v>-496420.253636</v>
+        <v>81229.05636399984</v>
       </c>
       <c r="R7" s="44" t="n">
-        <v>-529863.9321160002</v>
+        <v>47785.37788399961</v>
       </c>
       <c r="S7" s="44" t="n">
-        <v>-529863.9321160002</v>
+        <v>47785.37788399961</v>
       </c>
       <c r="T7" s="44" t="n">
-        <v>-529863.9321160002</v>
+        <v>47785.37788399961</v>
       </c>
       <c r="U7" s="44" t="n">
-        <v>-529863.9321160002</v>
+        <v>47785.37788399961</v>
       </c>
       <c r="V7" s="6" t="n"/>
       <c r="W7" s="6" t="n"/>
@@ -21659,61 +21635,61 @@
         <v>2006</v>
       </c>
       <c r="B8" s="44" t="n">
-        <v>980545.564728</v>
+        <v>805436.9647280001</v>
       </c>
       <c r="C8" s="44" t="n">
-        <v>588430.9509559998</v>
+        <v>413322.3509559999</v>
       </c>
       <c r="D8" s="44" t="n">
-        <v>739893.8076079998</v>
+        <v>564785.2076079999</v>
       </c>
       <c r="E8" s="44" t="n">
-        <v>669994.6483919998</v>
+        <v>494886.0483919999</v>
       </c>
       <c r="F8" s="44" t="n">
-        <v>660290.3891679998</v>
+        <v>485181.789168</v>
       </c>
       <c r="G8" s="44" t="n">
-        <v>605497.6544599999</v>
+        <v>430389.05446</v>
       </c>
       <c r="H8" s="44" t="n">
-        <v>555214.7979079997</v>
+        <v>380106.1979079999</v>
       </c>
       <c r="I8" s="44" t="n">
-        <v>577152.8443999998</v>
+        <v>402044.2444</v>
       </c>
       <c r="J8" s="44" t="n">
-        <v>546691.6862519998</v>
+        <v>371583.086252</v>
       </c>
       <c r="K8" s="44" t="n">
-        <v>502165.2547999998</v>
+        <v>327056.6547999999</v>
       </c>
       <c r="L8" s="44" t="n">
-        <v>398679.5835999998</v>
+        <v>223570.9835999999</v>
       </c>
       <c r="M8" s="44" t="n">
-        <v>317653.5043999997</v>
+        <v>142544.9043999999</v>
       </c>
       <c r="N8" s="44" t="n">
-        <v>278336.5634359997</v>
+        <v>103227.9634359998</v>
       </c>
       <c r="O8" s="44" t="n">
-        <v>262526.7261479993</v>
+        <v>87418.12614799943</v>
       </c>
       <c r="P8" s="44" t="n">
-        <v>261668.9861479993</v>
+        <v>86560.38614799944</v>
       </c>
       <c r="Q8" s="44" t="n">
-        <v>244514.1861479993</v>
+        <v>69405.58614799939</v>
       </c>
       <c r="R8" s="44" t="n">
-        <v>239895.5861479994</v>
+        <v>64786.98614799953</v>
       </c>
       <c r="S8" s="44" t="n">
-        <v>228894.1073399994</v>
+        <v>53785.50733999955</v>
       </c>
       <c r="T8" s="44" t="n">
-        <v>228894.1073399994</v>
+        <v>53785.50733999955</v>
       </c>
       <c r="U8" s="6" t="n"/>
       <c r="V8" s="6" t="n"/>
@@ -21726,58 +21702,58 @@
         <v>2007</v>
       </c>
       <c r="B9" s="44" t="n">
-        <v>1125681.558916</v>
+        <v>3213033.678915999</v>
       </c>
       <c r="C9" s="44" t="n">
-        <v>972575.8794399996</v>
+        <v>3059927.999439999</v>
       </c>
       <c r="D9" s="44" t="n">
-        <v>805231.6631799999</v>
+        <v>2892583.783179999</v>
       </c>
       <c r="E9" s="44" t="n">
-        <v>558909.5980559997</v>
+        <v>2646261.718055999</v>
       </c>
       <c r="F9" s="44" t="n">
-        <v>296146.9796279995</v>
+        <v>2383499.099627999</v>
       </c>
       <c r="G9" s="44" t="n">
-        <v>-198735.3373760004</v>
+        <v>1888616.782623999</v>
       </c>
       <c r="H9" s="44" t="n">
-        <v>-392696.0044000004</v>
+        <v>1694656.115599999</v>
       </c>
       <c r="I9" s="44" t="n">
-        <v>-747883.6443560002</v>
+        <v>1339468.475643999</v>
       </c>
       <c r="J9" s="44" t="n">
-        <v>-1005654.1632</v>
+        <v>1081697.956799999</v>
       </c>
       <c r="K9" s="44" t="n">
-        <v>-1397562.1672</v>
+        <v>689789.9527999992</v>
       </c>
       <c r="L9" s="44" t="n">
-        <v>-1527901.698400001</v>
+        <v>559450.4215999991</v>
       </c>
       <c r="M9" s="44" t="n">
-        <v>-1654399.174612001</v>
+        <v>432952.9453879986</v>
       </c>
       <c r="N9" s="44" t="n">
-        <v>-1726991.716603999</v>
+        <v>360360.4033960002</v>
       </c>
       <c r="O9" s="44" t="n">
-        <v>-1731261.612304</v>
+        <v>356090.5076959999</v>
       </c>
       <c r="P9" s="44" t="n">
-        <v>-1931130.260488</v>
+        <v>156221.8595119994</v>
       </c>
       <c r="Q9" s="44" t="n">
-        <v>-1931130.260488</v>
+        <v>156221.8595119994</v>
       </c>
       <c r="R9" s="44" t="n">
-        <v>-1948304.907271999</v>
+        <v>139047.2127280002</v>
       </c>
       <c r="S9" s="44" t="n">
-        <v>-1960436.174816</v>
+        <v>126915.9451839998</v>
       </c>
       <c r="T9" s="6" t="n"/>
       <c r="U9" s="6" t="n"/>
@@ -21791,55 +21767,55 @@
         <v>2008</v>
       </c>
       <c r="B10" s="44" t="n">
-        <v>1987574.162488</v>
+        <v>890344.7424879998</v>
       </c>
       <c r="C10" s="44" t="n">
-        <v>1773012.005832</v>
+        <v>675782.5858319999</v>
       </c>
       <c r="D10" s="44" t="n">
-        <v>1610761.181652</v>
+        <v>513531.7616519998</v>
       </c>
       <c r="E10" s="44" t="n">
-        <v>1245920.271816</v>
+        <v>148690.8518159997</v>
       </c>
       <c r="F10" s="44" t="n">
-        <v>1285807.93978</v>
+        <v>188578.5197799997</v>
       </c>
       <c r="G10" s="44" t="n">
-        <v>1264611.7988</v>
+        <v>167382.3787999998</v>
       </c>
       <c r="H10" s="44" t="n">
-        <v>1257683.133432</v>
+        <v>160453.7134319998</v>
       </c>
       <c r="I10" s="44" t="n">
-        <v>1240753.4308</v>
+        <v>143524.0107999998</v>
       </c>
       <c r="J10" s="44" t="n">
-        <v>1233305.6084</v>
+        <v>136076.1883999999</v>
       </c>
       <c r="K10" s="44" t="n">
-        <v>1187867.8216</v>
+        <v>90638.40159999975</v>
       </c>
       <c r="L10" s="44" t="n">
-        <v>1181195.026672</v>
+        <v>83965.60667199967</v>
       </c>
       <c r="M10" s="44" t="n">
-        <v>1180970.034872002</v>
+        <v>83740.61487200158</v>
       </c>
       <c r="N10" s="44" t="n">
-        <v>1200817.808572002</v>
+        <v>103588.3885720016</v>
       </c>
       <c r="O10" s="44" t="n">
-        <v>1200487.908572001</v>
+        <v>103258.4885720015</v>
       </c>
       <c r="P10" s="44" t="n">
-        <v>1200487.908572001</v>
+        <v>103258.4885720015</v>
       </c>
       <c r="Q10" s="44" t="n">
-        <v>1193889.908572001</v>
+        <v>96660.48857200146</v>
       </c>
       <c r="R10" s="44" t="n">
-        <v>1165499.110452001</v>
+        <v>68269.69045200152</v>
       </c>
       <c r="S10" s="6" t="n"/>
       <c r="T10" s="6" t="n"/>
@@ -21854,52 +21830,52 @@
         <v>2009</v>
       </c>
       <c r="B11" s="44" t="n">
-        <v>2237325.197828</v>
+        <v>891579.147828</v>
       </c>
       <c r="C11" s="44" t="n">
-        <v>1722268.136636</v>
+        <v>376522.086636</v>
       </c>
       <c r="D11" s="44" t="n">
-        <v>1772565.548376</v>
+        <v>426819.4983760001</v>
       </c>
       <c r="E11" s="44" t="n">
-        <v>1752051.666988</v>
+        <v>406305.616988</v>
       </c>
       <c r="F11" s="44" t="n">
-        <v>1696044.5044</v>
+        <v>350298.4543999999</v>
       </c>
       <c r="G11" s="44" t="n">
-        <v>1649915.959784</v>
+        <v>304169.909784</v>
       </c>
       <c r="H11" s="44" t="n">
-        <v>1615533.0692</v>
+        <v>269787.0192</v>
       </c>
       <c r="I11" s="44" t="n">
-        <v>1474451.994</v>
+        <v>128705.9439999999</v>
       </c>
       <c r="J11" s="44" t="n">
-        <v>1474445.396</v>
+        <v>128699.3459999999</v>
       </c>
       <c r="K11" s="44" t="n">
-        <v>1474443.693716</v>
+        <v>128697.6437159998</v>
       </c>
       <c r="L11" s="44" t="n">
-        <v>1474443.693715999</v>
+        <v>128697.6437159996</v>
       </c>
       <c r="M11" s="44" t="n">
-        <v>1459268.293715999</v>
+        <v>113522.2437159996</v>
       </c>
       <c r="N11" s="44" t="n">
-        <v>1425224.500743999</v>
+        <v>79478.45074399957</v>
       </c>
       <c r="O11" s="44" t="n">
-        <v>1425224.500743999</v>
+        <v>79478.45074399957</v>
       </c>
       <c r="P11" s="44" t="n">
-        <v>1425224.500743999</v>
+        <v>79478.45074399957</v>
       </c>
       <c r="Q11" s="44" t="n">
-        <v>1425224.500743999</v>
+        <v>79478.45074399957</v>
       </c>
       <c r="R11" s="6" t="n"/>
       <c r="S11" s="6" t="n"/>
@@ -21915,49 +21891,49 @@
         <v>2010</v>
       </c>
       <c r="B12" s="44" t="n">
-        <v>774270.290004</v>
+        <v>973394.130004</v>
       </c>
       <c r="C12" s="44" t="n">
-        <v>403710.3657279999</v>
+        <v>602834.205728</v>
       </c>
       <c r="D12" s="44" t="n">
-        <v>182978.6304079999</v>
+        <v>382102.4704079999</v>
       </c>
       <c r="E12" s="44" t="n">
-        <v>28962.86239999998</v>
+        <v>228086.7024000001</v>
       </c>
       <c r="F12" s="44" t="n">
-        <v>-101885.005112</v>
+        <v>97238.83488800004</v>
       </c>
       <c r="G12" s="44" t="n">
-        <v>-88598.98200000008</v>
+        <v>110524.858</v>
       </c>
       <c r="H12" s="44" t="n">
-        <v>-137066.5704000001</v>
+        <v>62057.2696</v>
       </c>
       <c r="I12" s="44" t="n">
-        <v>-138562.9968000001</v>
+        <v>60560.8432</v>
       </c>
       <c r="J12" s="44" t="n">
-        <v>-132521.326964</v>
+        <v>66602.51303600008</v>
       </c>
       <c r="K12" s="44" t="n">
-        <v>-133320.8066240004</v>
+        <v>65803.03337599966</v>
       </c>
       <c r="L12" s="44" t="n">
-        <v>-134315.7850240006</v>
+        <v>64808.05497599952</v>
       </c>
       <c r="M12" s="44" t="n">
-        <v>-134389.6826240006</v>
+        <v>64734.15737599949</v>
       </c>
       <c r="N12" s="44" t="n">
-        <v>-136039.1826240006</v>
+        <v>63084.65737599949</v>
       </c>
       <c r="O12" s="44" t="n">
-        <v>-135768.5326640005</v>
+        <v>63355.30733599956</v>
       </c>
       <c r="P12" s="44" t="n">
-        <v>-143371.3420840006</v>
+        <v>55752.4979159995</v>
       </c>
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="6" t="n"/>
@@ -21974,46 +21950,46 @@
         <v>2011</v>
       </c>
       <c r="B13" s="44" t="n">
-        <v>1088601.655408</v>
+        <v>1578461.035408</v>
       </c>
       <c r="C13" s="44" t="n">
-        <v>655729.229432</v>
+        <v>1145588.609432</v>
       </c>
       <c r="D13" s="44" t="n">
-        <v>234631.1191999998</v>
+        <v>724490.4992</v>
       </c>
       <c r="E13" s="44" t="n">
-        <v>32295.01695599989</v>
+        <v>522154.396956</v>
       </c>
       <c r="F13" s="44" t="n">
-        <v>-68890.07680000016</v>
+        <v>420969.3032</v>
       </c>
       <c r="G13" s="44" t="n">
-        <v>-197855.9044000001</v>
+        <v>292003.4756</v>
       </c>
       <c r="H13" s="44" t="n">
-        <v>-294053.4248000002</v>
+        <v>195805.9552</v>
       </c>
       <c r="I13" s="44" t="n">
-        <v>-294168.7050560003</v>
+        <v>195690.6749439999</v>
       </c>
       <c r="J13" s="44" t="n">
-        <v>-319494.4682559997</v>
+        <v>170364.9117440004</v>
       </c>
       <c r="K13" s="44" t="n">
-        <v>-326641.4218559996</v>
+        <v>163217.9581440005</v>
       </c>
       <c r="L13" s="44" t="n">
-        <v>-379336.9426759998</v>
+        <v>110522.4373240003</v>
       </c>
       <c r="M13" s="44" t="n">
-        <v>-373432.5904159998</v>
+        <v>116426.7895840004</v>
       </c>
       <c r="N13" s="44" t="n">
-        <v>-373432.5904159998</v>
+        <v>116426.7895840004</v>
       </c>
       <c r="O13" s="44" t="n">
-        <v>-373432.5904159998</v>
+        <v>116426.7895840004</v>
       </c>
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="6" t="n"/>
@@ -22031,43 +22007,43 @@
         <v>2012</v>
       </c>
       <c r="B14" s="44" t="n">
-        <v>1237614.865624</v>
+        <v>1126733.105624</v>
       </c>
       <c r="C14" s="44" t="n">
-        <v>891011.448</v>
+        <v>780129.688</v>
       </c>
       <c r="D14" s="44" t="n">
-        <v>681491.021084</v>
+        <v>570609.261084</v>
       </c>
       <c r="E14" s="44" t="n">
-        <v>604102.6963999999</v>
+        <v>493220.9363999999</v>
       </c>
       <c r="F14" s="44" t="n">
-        <v>607132.4979999999</v>
+        <v>496250.7379999999</v>
       </c>
       <c r="G14" s="44" t="n">
-        <v>598668.5835999999</v>
+        <v>487786.8235999999</v>
       </c>
       <c r="H14" s="44" t="n">
-        <v>594763.3065759999</v>
+        <v>483881.5465759999</v>
       </c>
       <c r="I14" s="44" t="n">
-        <v>544305.7613760012</v>
+        <v>433424.0013760012</v>
       </c>
       <c r="J14" s="44" t="n">
-        <v>486803.3732240011</v>
+        <v>375921.6132240011</v>
       </c>
       <c r="K14" s="44" t="n">
-        <v>425352.5967160012</v>
+        <v>314470.8367160012</v>
       </c>
       <c r="L14" s="44" t="n">
-        <v>416775.196716001</v>
+        <v>305893.436716001</v>
       </c>
       <c r="M14" s="44" t="n">
-        <v>209748.5894680009</v>
+        <v>98866.82946800091</v>
       </c>
       <c r="N14" s="44" t="n">
-        <v>209748.5894680009</v>
+        <v>98866.82946800091</v>
       </c>
       <c r="O14" s="6" t="n"/>
       <c r="P14" s="6" t="n"/>
@@ -22086,40 +22062,40 @@
         <v>2013</v>
       </c>
       <c r="B15" s="44" t="n">
-        <v>924632.2904000001</v>
+        <v>495460.1003999999</v>
       </c>
       <c r="C15" s="44" t="n">
-        <v>694072.860472</v>
+        <v>264900.6704719999</v>
       </c>
       <c r="D15" s="44" t="n">
-        <v>649607.8563999999</v>
+        <v>220435.6663999999</v>
       </c>
       <c r="E15" s="44" t="n">
-        <v>535680.1904</v>
+        <v>106508.0003999999</v>
       </c>
       <c r="F15" s="44" t="n">
-        <v>495082.6963999999</v>
+        <v>65910.50639999984</v>
       </c>
       <c r="G15" s="44" t="n">
-        <v>496924.3697479999</v>
+        <v>67752.17974799988</v>
       </c>
       <c r="H15" s="44" t="n">
-        <v>496575.8897800002</v>
+        <v>67403.69978000014</v>
       </c>
       <c r="I15" s="44" t="n">
-        <v>496575.88978</v>
+        <v>67403.69977999991</v>
       </c>
       <c r="J15" s="44" t="n">
-        <v>495210.2357400001</v>
+        <v>66038.04574000009</v>
       </c>
       <c r="K15" s="44" t="n">
-        <v>495210.2357400001</v>
+        <v>66038.04574000009</v>
       </c>
       <c r="L15" s="44" t="n">
-        <v>495199.0191400001</v>
+        <v>66026.82914000005</v>
       </c>
       <c r="M15" s="44" t="n">
-        <v>495199.0191400001</v>
+        <v>66026.82914000005</v>
       </c>
       <c r="N15" s="6" t="n"/>
       <c r="O15" s="6" t="n"/>
@@ -22139,37 +22115,37 @@
         <v>2014</v>
       </c>
       <c r="B16" s="44" t="n">
-        <v>648349.692516</v>
+        <v>946977.412516</v>
       </c>
       <c r="C16" s="44" t="n">
-        <v>436129.3640000001</v>
+        <v>734757.084</v>
       </c>
       <c r="D16" s="44" t="n">
-        <v>110314.8455999999</v>
+        <v>408942.5655999999</v>
       </c>
       <c r="E16" s="44" t="n">
-        <v>-64313.10080000013</v>
+        <v>234314.6191999998</v>
       </c>
       <c r="F16" s="44" t="n">
-        <v>-82786.35274800006</v>
+        <v>215841.3672519999</v>
       </c>
       <c r="G16" s="44" t="n">
-        <v>-127948.3431480001</v>
+        <v>170679.3768519999</v>
       </c>
       <c r="H16" s="44" t="n">
-        <v>-89131.50419200002</v>
+        <v>209496.2158079999</v>
       </c>
       <c r="I16" s="44" t="n">
-        <v>-89131.50419200002</v>
+        <v>209496.2158079999</v>
       </c>
       <c r="J16" s="44" t="n">
-        <v>-143235.1041920001</v>
+        <v>155392.6158079999</v>
       </c>
       <c r="K16" s="44" t="n">
-        <v>-171518.4340879999</v>
+        <v>127109.2859120001</v>
       </c>
       <c r="L16" s="44" t="n">
-        <v>-161800.094732</v>
+        <v>136827.6252679999</v>
       </c>
       <c r="M16" s="6" t="n"/>
       <c r="N16" s="6" t="n"/>
@@ -22190,34 +22166,34 @@
         <v>2015</v>
       </c>
       <c r="B17" s="44" t="n">
-        <v>1131745.98</v>
+        <v>3134339.12</v>
       </c>
       <c r="C17" s="44" t="n">
-        <v>601369.7087999999</v>
+        <v>2603962.8488</v>
       </c>
       <c r="D17" s="44" t="n">
-        <v>64210.69359999965</v>
+        <v>2066803.8336</v>
       </c>
       <c r="E17" s="44" t="n">
-        <v>-463210.3597920001</v>
+        <v>1539382.780208</v>
       </c>
       <c r="F17" s="44" t="n">
-        <v>-689151.6779720015</v>
+        <v>1313441.462027999</v>
       </c>
       <c r="G17" s="44" t="n">
-        <v>-1010457.255132001</v>
+        <v>992135.8848679988</v>
       </c>
       <c r="H17" s="44" t="n">
-        <v>-1385520.525544002</v>
+        <v>617072.6144559984</v>
       </c>
       <c r="I17" s="44" t="n">
-        <v>-1406238.245544002</v>
+        <v>596354.8944559982</v>
       </c>
       <c r="J17" s="44" t="n">
-        <v>-1416392.290428002</v>
+        <v>586200.8495719982</v>
       </c>
       <c r="K17" s="44" t="n">
-        <v>-1713150.378076002</v>
+        <v>289442.7619239986</v>
       </c>
       <c r="L17" s="6" t="n"/>
       <c r="M17" s="6" t="n"/>
@@ -22239,31 +22215,31 @@
         <v>2016</v>
       </c>
       <c r="B18" s="44" t="n">
-        <v>1867011.798</v>
+        <v>2243886.108</v>
       </c>
       <c r="C18" s="44" t="n">
-        <v>1268852.9532</v>
+        <v>1645727.2632</v>
       </c>
       <c r="D18" s="44" t="n">
-        <v>821343.721964</v>
+        <v>1198218.031964</v>
       </c>
       <c r="E18" s="44" t="n">
-        <v>670546.0888680003</v>
+        <v>1047420.398868</v>
       </c>
       <c r="F18" s="44" t="n">
-        <v>402397.7473720009</v>
+        <v>779272.057372001</v>
       </c>
       <c r="G18" s="44" t="n">
-        <v>334396.2257400011</v>
+        <v>711270.5357400011</v>
       </c>
       <c r="H18" s="44" t="n">
-        <v>51193.24084000103</v>
+        <v>428067.5508400011</v>
       </c>
       <c r="I18" s="44" t="n">
-        <v>51789.0666320012</v>
+        <v>428663.3766320013</v>
       </c>
       <c r="J18" s="44" t="n">
-        <v>48490.0666320012</v>
+        <v>425364.3766320013</v>
       </c>
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="6" t="n"/>
@@ -22286,28 +22262,28 @@
         <v>2017</v>
       </c>
       <c r="B19" s="44" t="n">
-        <v>2144583.1084</v>
+        <v>1081527.6484</v>
       </c>
       <c r="C19" s="44" t="n">
-        <v>1991037.302736</v>
+        <v>927981.842736</v>
       </c>
       <c r="D19" s="44" t="n">
-        <v>1969910.783852</v>
+        <v>906855.3238519996</v>
       </c>
       <c r="E19" s="44" t="n">
-        <v>1773139.777904</v>
+        <v>710084.3179039995</v>
       </c>
       <c r="F19" s="44" t="n">
-        <v>1710620.50808</v>
+        <v>647565.0480799995</v>
       </c>
       <c r="G19" s="44" t="n">
-        <v>1591801.691896</v>
+        <v>528746.2318959996</v>
       </c>
       <c r="H19" s="44" t="n">
-        <v>1436957.096324</v>
+        <v>373901.6363239996</v>
       </c>
       <c r="I19" s="44" t="n">
-        <v>1400098.161084</v>
+        <v>337042.7010839996</v>
       </c>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
@@ -22331,25 +22307,25 @@
         <v>2018</v>
       </c>
       <c r="B20" s="44" t="n">
-        <v>1707039.669552</v>
+        <v>2328567.799552</v>
       </c>
       <c r="C20" s="44" t="n">
-        <v>1046955.572868</v>
+        <v>1668483.702868</v>
       </c>
       <c r="D20" s="44" t="n">
-        <v>546165.2879000008</v>
+        <v>1167693.417900001</v>
       </c>
       <c r="E20" s="44" t="n">
-        <v>-101796.1450320007</v>
+        <v>519731.9849679992</v>
       </c>
       <c r="F20" s="44" t="n">
-        <v>-88494.61662000045</v>
+        <v>533033.5133799994</v>
       </c>
       <c r="G20" s="44" t="n">
-        <v>-118651.8576920005</v>
+        <v>502876.2723079994</v>
       </c>
       <c r="H20" s="44" t="n">
-        <v>-180424.9333040006</v>
+        <v>441103.1966959992</v>
       </c>
       <c r="I20" s="6" t="n"/>
       <c r="J20" s="6" t="n"/>
@@ -22374,22 +22350,22 @@
         <v>2019</v>
       </c>
       <c r="B21" s="44" t="n">
-        <v>1851409.128824</v>
+        <v>2869721.688824</v>
       </c>
       <c r="C21" s="44" t="n">
-        <v>1134716.89732</v>
+        <v>2153029.45732</v>
       </c>
       <c r="D21" s="44" t="n">
-        <v>519269.4186879995</v>
+        <v>1537581.978688</v>
       </c>
       <c r="E21" s="44" t="n">
-        <v>258760.9145879999</v>
+        <v>1277073.474588</v>
       </c>
       <c r="F21" s="44" t="n">
-        <v>131945.2696199999</v>
+        <v>1150257.82962</v>
       </c>
       <c r="G21" s="44" t="n">
-        <v>-340558.9142919993</v>
+        <v>677753.6457080008</v>
       </c>
       <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="n"/>
@@ -22415,19 +22391,19 @@
         <v>2020</v>
       </c>
       <c r="B22" s="44" t="n">
-        <v>1321505.746468</v>
+        <v>961951.9364680001</v>
       </c>
       <c r="C22" s="44" t="n">
-        <v>911692.8290440004</v>
+        <v>552139.0190440003</v>
       </c>
       <c r="D22" s="44" t="n">
-        <v>927316.5499480002</v>
+        <v>567762.7399480002</v>
       </c>
       <c r="E22" s="44" t="n">
-        <v>874140.0481240002</v>
+        <v>514586.2381240001</v>
       </c>
       <c r="F22" s="44" t="n">
-        <v>864708.8405320002</v>
+        <v>505155.0305320001</v>
       </c>
       <c r="G22" s="6" t="n"/>
       <c r="H22" s="6" t="n"/>
@@ -22454,16 +22430,16 @@
         <v>2021</v>
       </c>
       <c r="B23" s="44" t="n">
-        <v>860903.3230120001</v>
+        <v>965231.1130120001</v>
       </c>
       <c r="C23" s="44" t="n">
-        <v>609425.2375919998</v>
+        <v>713753.0275919999</v>
       </c>
       <c r="D23" s="44" t="n">
-        <v>430043.6037400002</v>
+        <v>534371.3937400002</v>
       </c>
       <c r="E23" s="44" t="n">
-        <v>399047.1102639999</v>
+        <v>503374.9002639999</v>
       </c>
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="n"/>
@@ -22491,13 +22467,13 @@
         <v>2022</v>
       </c>
       <c r="B24" s="44" t="n">
-        <v>264422.056424</v>
+        <v>689813.846424</v>
       </c>
       <c r="C24" s="44" t="n">
-        <v>107389.1813679991</v>
+        <v>532780.9713679991</v>
       </c>
       <c r="D24" s="44" t="n">
-        <v>131628.9533559993</v>
+        <v>557020.7433559994</v>
       </c>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
@@ -22526,10 +22502,10 @@
         <v>2023</v>
       </c>
       <c r="B25" s="44" t="n">
-        <v>3225.657395999762</v>
+        <v>1228284.677396</v>
       </c>
       <c r="C25" s="44" t="n">
-        <v>-673530.7143519998</v>
+        <v>551528.3056480002</v>
       </c>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="n"/>
@@ -22559,7 +22535,7 @@
         <v>2024</v>
       </c>
       <c r="B26" s="44" t="n">
-        <v>107635.2581719999</v>
+        <v>424884.038172</v>
       </c>
       <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>

</xml_diff>